<commit_message>
Demo grades on one company-wide ladder
Each category's grades are shifted by a constant onto a single 1-12 ladder
(higher number = more senior), so no office role starts at grade 1:
Customer Support 3-6, Manufacturing 4-8, Operations 5-10, Marketing 6-10,
Engineering 7-12, Sales 8-12, Legal 9-12. Range widths are unchanged, so
salaries, tenure and every result stay the same (EUR 148,426 / 396,245);
only the regression intercept moves. Wider helper columns on the
Categories sheet so the larger regression sums display.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JrJSoh7gpksFWuaoBdtVSD
</commit_message>
<xml_diff>
--- a/pay-gap-calculator/pay-gap-model.xlsx
+++ b/pay-gap-calculator/pay-gap-model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Projects IA\PROJECT-pay-gap-calculator\pay-gap-calculator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DC8C47B-7131-4D97-BB75-2CCD834AEEB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD473A0A-1449-4564-A76C-0530419C64C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2113,7 +2113,7 @@
         <v>5.6</v>
       </c>
       <c r="G5" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H5" s="8">
         <v>1</v>
@@ -2238,7 +2238,7 @@
         <v>8.9</v>
       </c>
       <c r="G6" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H6" s="8">
         <v>1</v>
@@ -2363,7 +2363,7 @@
         <v>11.8</v>
       </c>
       <c r="G7" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H7" s="8">
         <v>1</v>
@@ -2488,7 +2488,7 @@
         <v>7.4</v>
       </c>
       <c r="G8" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H8" s="8">
         <v>1</v>
@@ -2613,7 +2613,7 @@
         <v>6.6</v>
       </c>
       <c r="G9" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H9" s="8">
         <v>1</v>
@@ -2738,7 +2738,7 @@
         <v>5.5</v>
       </c>
       <c r="G10" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H10" s="8">
         <v>1</v>
@@ -2863,7 +2863,7 @@
         <v>4.8</v>
       </c>
       <c r="G11" s="8">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H11" s="8">
         <v>1</v>
@@ -2988,7 +2988,7 @@
         <v>6.6</v>
       </c>
       <c r="G12" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H12" s="8">
         <v>1</v>
@@ -3113,7 +3113,7 @@
         <v>5.9</v>
       </c>
       <c r="G13" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H13" s="8">
         <v>1</v>
@@ -3238,7 +3238,7 @@
         <v>9.6999999999999993</v>
       </c>
       <c r="G14" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H14" s="8">
         <v>1</v>
@@ -3363,7 +3363,7 @@
         <v>2.8</v>
       </c>
       <c r="G15" s="8">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H15" s="8">
         <v>1</v>
@@ -3488,7 +3488,7 @@
         <v>7.7</v>
       </c>
       <c r="G16" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H16" s="8">
         <v>1</v>
@@ -3613,7 +3613,7 @@
         <v>7.6</v>
       </c>
       <c r="G17" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H17" s="8">
         <v>0.6</v>
@@ -3659,19 +3659,19 @@
       </c>
       <c r="S17" s="11">
         <f>R17*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B17)</f>
-        <v>4097.1936535686154</v>
+        <v>4097.1936535686264</v>
       </c>
       <c r="T17" s="11">
         <f t="shared" si="7"/>
-        <v>2458.3161921411693</v>
+        <v>2458.3161921411756</v>
       </c>
       <c r="U17" s="11">
         <f t="shared" si="8"/>
-        <v>774.3696005244683</v>
+        <v>774.36960052447034</v>
       </c>
       <c r="V17" s="11">
         <f t="shared" si="9"/>
-        <v>3232.6857926656376</v>
+        <v>3232.6857926656457</v>
       </c>
       <c r="W17" s="12">
         <f>IF(AND(C17="F",M17&lt;O17,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B17)=1),1,0)</f>
@@ -3687,19 +3687,19 @@
       </c>
       <c r="Z17" s="11">
         <f>Y17*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B17)</f>
-        <v>9118.2318849490221</v>
+        <v>9118.2318849490348</v>
       </c>
       <c r="AA17" s="11">
         <f t="shared" si="11"/>
-        <v>5470.9391309694129</v>
+        <v>5470.9391309694211</v>
       </c>
       <c r="AB17" s="11">
         <f t="shared" si="12"/>
-        <v>1723.345826255365</v>
+        <v>1723.3458262553677</v>
       </c>
       <c r="AC17" s="11">
         <f t="shared" si="13"/>
-        <v>7194.2849572247778</v>
+        <v>7194.2849572247887</v>
       </c>
       <c r="AD17" s="12">
         <f t="shared" si="14"/>
@@ -3738,7 +3738,7 @@
         <v>7.8</v>
       </c>
       <c r="G18" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H18" s="8">
         <v>1</v>
@@ -3863,7 +3863,7 @@
         <v>9.9</v>
       </c>
       <c r="G19" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H19" s="8">
         <v>1</v>
@@ -3909,19 +3909,19 @@
       </c>
       <c r="S19" s="11">
         <f>R19*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B19)</f>
-        <v>93.377951954064955</v>
+        <v>93.377951954065196</v>
       </c>
       <c r="T19" s="11">
         <f t="shared" si="7"/>
-        <v>93.377951954064955</v>
+        <v>93.377951954065196</v>
       </c>
       <c r="U19" s="11">
         <f t="shared" si="8"/>
-        <v>0.8964283387590235</v>
+        <v>0.89642833875902583</v>
       </c>
       <c r="V19" s="11">
         <f t="shared" si="9"/>
-        <v>94.274380292823977</v>
+        <v>94.274380292824219</v>
       </c>
       <c r="W19" s="12">
         <f>IF(AND(C19="F",M19&lt;O19,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B19)=1),1,0)</f>
@@ -3937,19 +3937,19 @@
       </c>
       <c r="Z19" s="11">
         <f>Y19*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B19)</f>
-        <v>207.81097767180114</v>
+        <v>207.8109776718014</v>
       </c>
       <c r="AA19" s="11">
         <f t="shared" si="11"/>
-        <v>207.81097767180114</v>
+        <v>207.8109776718014</v>
       </c>
       <c r="AB19" s="11">
         <f t="shared" si="12"/>
-        <v>1.9949853856492907</v>
+        <v>1.9949853856492932</v>
       </c>
       <c r="AC19" s="11">
         <f t="shared" si="13"/>
-        <v>209.80596305745044</v>
+        <v>209.8059630574507</v>
       </c>
       <c r="AD19" s="12">
         <f t="shared" si="14"/>
@@ -3988,7 +3988,7 @@
         <v>7.2</v>
       </c>
       <c r="G20" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H20" s="8">
         <v>1</v>
@@ -4034,19 +4034,19 @@
       </c>
       <c r="S20" s="11">
         <f>R20*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B20)</f>
-        <v>3498.7659362173204</v>
+        <v>3498.7659362173295</v>
       </c>
       <c r="T20" s="11">
         <f t="shared" si="7"/>
-        <v>3498.7659362173204</v>
+        <v>3498.7659362173295</v>
       </c>
       <c r="U20" s="11">
         <f t="shared" si="8"/>
-        <v>1102.1112699084558</v>
+        <v>1102.1112699084588</v>
       </c>
       <c r="V20" s="11">
         <f t="shared" si="9"/>
-        <v>4600.877206125776</v>
+        <v>4600.8772061257878</v>
       </c>
       <c r="W20" s="12">
         <f>IF(AND(C20="F",M20&lt;O20,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B20)=1),1,0)</f>
@@ -4062,11 +4062,11 @@
       </c>
       <c r="Z20" s="11">
         <f>Y20*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B20)</f>
-        <v>7786.4416024864904</v>
+        <v>7786.4416024865004</v>
       </c>
       <c r="AA20" s="11">
         <f t="shared" si="11"/>
-        <v>7786.4416024864904</v>
+        <v>7786.4416024865004</v>
       </c>
       <c r="AB20" s="11">
         <f t="shared" si="12"/>
@@ -4074,7 +4074,7 @@
       </c>
       <c r="AC20" s="11">
         <f t="shared" si="13"/>
-        <v>9051.063435870361</v>
+        <v>9051.0634358703719</v>
       </c>
       <c r="AD20" s="12">
         <f t="shared" si="14"/>
@@ -4113,7 +4113,7 @@
         <v>0.6</v>
       </c>
       <c r="G21" s="8">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H21" s="8">
         <v>1</v>
@@ -4159,19 +4159,19 @@
       </c>
       <c r="S21" s="11">
         <f>R21*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B21)</f>
-        <v>8749.6943934172305</v>
+        <v>8749.6943934172541</v>
       </c>
       <c r="T21" s="11">
         <f t="shared" si="7"/>
-        <v>8749.6943934172305</v>
+        <v>8749.6943934172541</v>
       </c>
       <c r="U21" s="11">
         <f t="shared" si="8"/>
-        <v>2756.1537339264278</v>
+        <v>2756.1537339264351</v>
       </c>
       <c r="V21" s="11">
         <f t="shared" si="9"/>
-        <v>11505.848127343659</v>
+        <v>11505.848127343688</v>
       </c>
       <c r="W21" s="12">
         <f>IF(AND(C21="F",M21&lt;O21,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B21)=1),1,0)</f>
@@ -4187,19 +4187,19 @@
       </c>
       <c r="Z21" s="11">
         <f>Y21*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B21)</f>
-        <v>19472.289851891081</v>
+        <v>19472.289851891106</v>
       </c>
       <c r="AA21" s="11">
         <f t="shared" si="11"/>
-        <v>19472.289851891081</v>
+        <v>19472.289851891106</v>
       </c>
       <c r="AB21" s="11">
         <f t="shared" si="12"/>
-        <v>5611.9343685781532</v>
+        <v>5611.9343685781541</v>
       </c>
       <c r="AC21" s="11">
         <f t="shared" si="13"/>
-        <v>25084.224220469234</v>
+        <v>25084.224220469259</v>
       </c>
       <c r="AD21" s="12">
         <f t="shared" si="14"/>
@@ -4238,7 +4238,7 @@
         <v>10.199999999999999</v>
       </c>
       <c r="G22" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H22" s="8">
         <v>1</v>
@@ -4363,7 +4363,7 @@
         <v>11.6</v>
       </c>
       <c r="G23" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H23" s="8">
         <v>1</v>
@@ -4488,7 +4488,7 @@
         <v>9.6</v>
       </c>
       <c r="G24" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H24" s="8">
         <v>1</v>
@@ -4613,7 +4613,7 @@
         <v>5.9</v>
       </c>
       <c r="G25" s="8">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H25" s="8">
         <v>1</v>
@@ -4738,7 +4738,7 @@
         <v>0.7</v>
       </c>
       <c r="G26" s="8">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H26" s="8">
         <v>1</v>
@@ -4863,7 +4863,7 @@
         <v>6</v>
       </c>
       <c r="G27" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H27" s="8">
         <v>1</v>
@@ -4988,7 +4988,7 @@
         <v>4.8</v>
       </c>
       <c r="G28" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H28" s="8">
         <v>1</v>
@@ -5113,7 +5113,7 @@
         <v>4.8</v>
       </c>
       <c r="G29" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H29" s="8">
         <v>1</v>
@@ -5238,7 +5238,7 @@
         <v>7</v>
       </c>
       <c r="G30" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H30" s="8">
         <v>1</v>
@@ -5284,11 +5284,11 @@
       </c>
       <c r="S30" s="11">
         <f>R30*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B30)</f>
-        <v>1369.3166741234686</v>
+        <v>1369.3166741234722</v>
       </c>
       <c r="T30" s="11">
         <f t="shared" si="7"/>
-        <v>1369.3166741234686</v>
+        <v>1369.3166741234722</v>
       </c>
       <c r="U30" s="11">
         <f t="shared" si="8"/>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="V30" s="11">
         <f t="shared" si="9"/>
-        <v>1700.6889141950539</v>
+        <v>1700.6889141950576</v>
       </c>
       <c r="W30" s="12">
         <f>IF(AND(C30="F",M30&lt;O30,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B30)=1),1,0)</f>
@@ -5312,19 +5312,19 @@
       </c>
       <c r="Z30" s="11">
         <f>Y30*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B30)</f>
-        <v>3047.3899977146548</v>
+        <v>3047.3899977146589</v>
       </c>
       <c r="AA30" s="11">
         <f t="shared" si="11"/>
-        <v>3047.3899977146548</v>
+        <v>3047.3899977146589</v>
       </c>
       <c r="AB30" s="11">
         <f t="shared" si="12"/>
-        <v>347.48174397806071</v>
+        <v>347.48174397806076</v>
       </c>
       <c r="AC30" s="11">
         <f t="shared" si="13"/>
-        <v>3394.8717416927157</v>
+        <v>3394.8717416927198</v>
       </c>
       <c r="AD30" s="12">
         <f t="shared" si="14"/>
@@ -5363,7 +5363,7 @@
         <v>4.8</v>
       </c>
       <c r="G31" s="8">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H31" s="8">
         <v>1</v>
@@ -5488,7 +5488,7 @@
         <v>4.2</v>
       </c>
       <c r="G32" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H32" s="8">
         <v>1</v>
@@ -5534,19 +5534,19 @@
       </c>
       <c r="S32" s="11">
         <f>R32*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B32)</f>
-        <v>6089.6435122994544</v>
+        <v>6089.6435122994708</v>
       </c>
       <c r="T32" s="11">
         <f t="shared" si="7"/>
-        <v>6089.6435122994544</v>
+        <v>6089.6435122994708</v>
       </c>
       <c r="U32" s="11">
         <f t="shared" si="8"/>
-        <v>1918.2377063743281</v>
+        <v>1918.2377063743334</v>
       </c>
       <c r="V32" s="11">
         <f t="shared" si="9"/>
-        <v>8007.8812186737823</v>
+        <v>8007.8812186738041</v>
       </c>
       <c r="W32" s="12">
         <f>IF(AND(C32="F",M32&lt;O32,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B32)=1),1,0)</f>
@@ -5562,19 +5562,19 @@
       </c>
       <c r="Z32" s="11">
         <f>Y32*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B32)</f>
-        <v>13552.393744791281</v>
+        <v>13552.393744791299</v>
       </c>
       <c r="AA32" s="11">
         <f t="shared" si="11"/>
-        <v>13552.393744791281</v>
+        <v>13552.393744791299</v>
       </c>
       <c r="AB32" s="11">
         <f t="shared" si="12"/>
-        <v>3273.8569859499958</v>
+        <v>3273.8569859499962</v>
       </c>
       <c r="AC32" s="11">
         <f t="shared" si="13"/>
-        <v>16826.250730741278</v>
+        <v>16826.250730741296</v>
       </c>
       <c r="AD32" s="12">
         <f t="shared" si="14"/>
@@ -5613,7 +5613,7 @@
         <v>8.3000000000000007</v>
       </c>
       <c r="G33" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H33" s="8">
         <v>1</v>
@@ -5738,7 +5738,7 @@
         <v>8.4</v>
       </c>
       <c r="G34" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H34" s="8">
         <v>1</v>
@@ -5863,7 +5863,7 @@
         <v>7.4</v>
       </c>
       <c r="G35" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H35" s="8">
         <v>1</v>
@@ -5988,7 +5988,7 @@
         <v>10.1</v>
       </c>
       <c r="G36" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H36" s="8">
         <v>1</v>
@@ -6113,7 +6113,7 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="G37" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H37" s="8">
         <v>1</v>
@@ -6238,7 +6238,7 @@
         <v>7.7</v>
       </c>
       <c r="G38" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H38" s="8">
         <v>1</v>
@@ -6363,7 +6363,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="G39" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H39" s="8">
         <v>1</v>
@@ -6488,7 +6488,7 @@
         <v>9.9</v>
       </c>
       <c r="G40" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H40" s="8">
         <v>1</v>
@@ -6613,7 +6613,7 @@
         <v>11</v>
       </c>
       <c r="G41" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H41" s="8">
         <v>1</v>
@@ -6738,7 +6738,7 @@
         <v>4.9000000000000004</v>
       </c>
       <c r="G42" s="8">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H42" s="8">
         <v>1</v>
@@ -6784,19 +6784,19 @@
       </c>
       <c r="S42" s="11">
         <f>R42*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B42)</f>
-        <v>8600.2370841552765</v>
+        <v>8600.2370841553002</v>
       </c>
       <c r="T42" s="11">
         <f t="shared" si="7"/>
-        <v>8600.2370841552765</v>
+        <v>8600.2370841553002</v>
       </c>
       <c r="U42" s="11">
         <f t="shared" si="8"/>
-        <v>2709.0746815089119</v>
+        <v>2709.0746815089196</v>
       </c>
       <c r="V42" s="11">
         <f t="shared" si="9"/>
-        <v>11309.311765664188</v>
+        <v>11309.311765664221</v>
       </c>
       <c r="W42" s="12">
         <f>IF(AND(C42="F",M42&lt;O42,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B42)=1),1,0)</f>
@@ -6812,11 +6812,11 @@
       </c>
       <c r="Z42" s="11">
         <f>Y42*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B42)</f>
-        <v>19139.675258103438</v>
+        <v>19139.675258103463</v>
       </c>
       <c r="AA42" s="11">
         <f t="shared" si="11"/>
-        <v>19139.675258103438</v>
+        <v>19139.675258103463</v>
       </c>
       <c r="AB42" s="11">
         <f t="shared" si="12"/>
@@ -6824,7 +6824,7 @@
       </c>
       <c r="AC42" s="11">
         <f t="shared" si="13"/>
-        <v>24812.70322658123</v>
+        <v>24812.703226581256</v>
       </c>
       <c r="AD42" s="12">
         <f t="shared" si="14"/>
@@ -6863,7 +6863,7 @@
         <v>3.6</v>
       </c>
       <c r="G43" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H43" s="8">
         <v>1</v>
@@ -6909,19 +6909,19 @@
       </c>
       <c r="S43" s="11">
         <f>R43*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B43)</f>
-        <v>4069.3442866429787</v>
+        <v>4069.3442866429891</v>
       </c>
       <c r="T43" s="11">
         <f t="shared" si="7"/>
-        <v>4069.3442866429787</v>
+        <v>4069.3442866429891</v>
       </c>
       <c r="U43" s="11">
         <f t="shared" si="8"/>
-        <v>1281.8434502925384</v>
+        <v>1281.8434502925415</v>
       </c>
       <c r="V43" s="11">
         <f t="shared" si="9"/>
-        <v>5351.187736935517</v>
+        <v>5351.1877369355307</v>
       </c>
       <c r="W43" s="12">
         <f>IF(AND(C43="F",M43&lt;O43,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B43)=1),1,0)</f>
@@ -6937,19 +6937,19 @@
       </c>
       <c r="Z43" s="11">
         <f>Y43*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B43)</f>
-        <v>9056.253612270646</v>
+        <v>9056.2536122706588</v>
       </c>
       <c r="AA43" s="11">
         <f t="shared" si="11"/>
-        <v>9056.253612270646</v>
+        <v>9056.2536122706588</v>
       </c>
       <c r="AB43" s="11">
         <f t="shared" si="12"/>
-        <v>2364.4238866777973</v>
+        <v>2364.4238866777978</v>
       </c>
       <c r="AC43" s="11">
         <f t="shared" si="13"/>
-        <v>11420.677498948444</v>
+        <v>11420.677498948457</v>
       </c>
       <c r="AD43" s="12">
         <f t="shared" si="14"/>
@@ -6988,7 +6988,7 @@
         <v>10.199999999999999</v>
       </c>
       <c r="G44" s="8">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H44" s="8">
         <v>1</v>
@@ -7113,7 +7113,7 @@
         <v>4.8</v>
       </c>
       <c r="G45" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H45" s="8">
         <v>1</v>
@@ -7238,7 +7238,7 @@
         <v>11</v>
       </c>
       <c r="G46" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H46" s="8">
         <v>1</v>
@@ -7363,7 +7363,7 @@
         <v>7.2</v>
       </c>
       <c r="G47" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H47" s="8">
         <v>1</v>
@@ -7488,7 +7488,7 @@
         <v>7.7</v>
       </c>
       <c r="G48" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H48" s="8">
         <v>1</v>
@@ -7613,7 +7613,7 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="G49" s="8">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H49" s="8">
         <v>1</v>
@@ -7738,7 +7738,7 @@
         <v>5.5</v>
       </c>
       <c r="G50" s="8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H50" s="8">
         <v>1</v>
@@ -7863,7 +7863,7 @@
         <v>5.6</v>
       </c>
       <c r="G51" s="8">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H51" s="8">
         <v>0.6</v>
@@ -7988,7 +7988,7 @@
         <v>9.6999999999999993</v>
       </c>
       <c r="G52" s="8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H52" s="8">
         <v>1</v>
@@ -8113,7 +8113,7 @@
         <v>9.9</v>
       </c>
       <c r="G53" s="8">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H53" s="8">
         <v>1</v>
@@ -8238,7 +8238,7 @@
         <v>4</v>
       </c>
       <c r="G54" s="8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H54" s="8">
         <v>1</v>
@@ -8363,7 +8363,7 @@
         <v>6.6</v>
       </c>
       <c r="G55" s="8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H55" s="8">
         <v>1</v>
@@ -8488,7 +8488,7 @@
         <v>5.3</v>
       </c>
       <c r="G56" s="8">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H56" s="8">
         <v>1</v>
@@ -8613,7 +8613,7 @@
         <v>4.5</v>
       </c>
       <c r="G57" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H57" s="8">
         <v>1</v>
@@ -8738,7 +8738,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="G58" s="8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H58" s="8">
         <v>1</v>
@@ -8812,19 +8812,19 @@
       </c>
       <c r="Z58" s="11">
         <f>Y58*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B58)</f>
-        <v>1172.2428068588774</v>
+        <v>1172.2428068588972</v>
       </c>
       <c r="AA58" s="11">
         <f t="shared" si="11"/>
-        <v>1172.2428068588774</v>
+        <v>1172.2428068588972</v>
       </c>
       <c r="AB58" s="11">
         <f t="shared" si="12"/>
-        <v>369.25648416054639</v>
+        <v>369.25648416055265</v>
       </c>
       <c r="AC58" s="11">
         <f t="shared" si="13"/>
-        <v>1541.4992910194237</v>
+        <v>1541.4992910194499</v>
       </c>
       <c r="AD58" s="12">
         <f t="shared" si="14"/>
@@ -8863,7 +8863,7 @@
         <v>5.9</v>
       </c>
       <c r="G59" s="8">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H59" s="8">
         <v>1</v>
@@ -8988,7 +8988,7 @@
         <v>3</v>
       </c>
       <c r="G60" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H60" s="8">
         <v>1</v>
@@ -9062,19 +9062,19 @@
       </c>
       <c r="Z60" s="11">
         <f>Y60*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B60)</f>
-        <v>1342.0753160669174</v>
+        <v>1342.0753160669401</v>
       </c>
       <c r="AA60" s="11">
         <f t="shared" si="11"/>
-        <v>1342.0753160669174</v>
+        <v>1342.0753160669401</v>
       </c>
       <c r="AB60" s="11">
         <f t="shared" si="12"/>
-        <v>422.75372456107897</v>
+        <v>422.75372456108613</v>
       </c>
       <c r="AC60" s="11">
         <f t="shared" si="13"/>
-        <v>1764.8290406279964</v>
+        <v>1764.8290406280262</v>
       </c>
       <c r="AD60" s="12">
         <f t="shared" si="14"/>
@@ -9113,7 +9113,7 @@
         <v>6.4</v>
       </c>
       <c r="G61" s="8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H61" s="8">
         <v>1</v>
@@ -9238,7 +9238,7 @@
         <v>9.9</v>
       </c>
       <c r="G62" s="8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H62" s="8">
         <v>0.8</v>
@@ -9363,7 +9363,7 @@
         <v>9.1</v>
       </c>
       <c r="G63" s="8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H63" s="8">
         <v>1</v>
@@ -9488,7 +9488,7 @@
         <v>1.6</v>
       </c>
       <c r="G64" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H64" s="8">
         <v>1</v>
@@ -9562,19 +9562,19 @@
       </c>
       <c r="Z64" s="11">
         <f>Y64*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B64)</f>
-        <v>1283.7918127908749</v>
+        <v>1283.7918127908965</v>
       </c>
       <c r="AA64" s="11">
         <f t="shared" si="11"/>
-        <v>1283.7918127908749</v>
+        <v>1283.7918127908965</v>
       </c>
       <c r="AB64" s="11">
         <f t="shared" si="12"/>
-        <v>404.39442102912562</v>
+        <v>404.39442102913239</v>
       </c>
       <c r="AC64" s="11">
         <f t="shared" si="13"/>
-        <v>1688.1862338200006</v>
+        <v>1688.186233820029</v>
       </c>
       <c r="AD64" s="12">
         <f t="shared" si="14"/>
@@ -9613,7 +9613,7 @@
         <v>4.2</v>
       </c>
       <c r="G65" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H65" s="8">
         <v>1</v>
@@ -9687,19 +9687,19 @@
       </c>
       <c r="Z65" s="11">
         <f>Y65*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B65)</f>
-        <v>1834.3550539225441</v>
+        <v>1834.3550539225748</v>
       </c>
       <c r="AA65" s="11">
         <f t="shared" si="11"/>
-        <v>1834.3550539225441</v>
+        <v>1834.3550539225748</v>
       </c>
       <c r="AB65" s="11">
         <f t="shared" si="12"/>
-        <v>577.8218419856014</v>
+        <v>577.82184198561106</v>
       </c>
       <c r="AC65" s="11">
         <f t="shared" si="13"/>
-        <v>2412.1768959081455</v>
+        <v>2412.176895908186</v>
       </c>
       <c r="AD65" s="12">
         <f t="shared" si="14"/>
@@ -9738,7 +9738,7 @@
         <v>7.7</v>
       </c>
       <c r="G66" s="8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H66" s="8">
         <v>1</v>
@@ -9863,7 +9863,7 @@
         <v>2.1</v>
       </c>
       <c r="G67" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H67" s="8">
         <v>1</v>
@@ -9937,19 +9937,19 @@
       </c>
       <c r="Z67" s="11">
         <f>Y67*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B67)</f>
-        <v>1971.927763992197</v>
+        <v>1971.9277639922302</v>
       </c>
       <c r="AA67" s="11">
         <f t="shared" si="11"/>
-        <v>1971.927763992197</v>
+        <v>1971.9277639922302</v>
       </c>
       <c r="AB67" s="11">
         <f t="shared" si="12"/>
-        <v>621.15724565754203</v>
+        <v>621.15724565755249</v>
       </c>
       <c r="AC67" s="11">
         <f t="shared" si="13"/>
-        <v>2593.0850096497388</v>
+        <v>2593.0850096497825</v>
       </c>
       <c r="AD67" s="12">
         <f t="shared" si="14"/>
@@ -9988,7 +9988,7 @@
         <v>1.9</v>
       </c>
       <c r="G68" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H68" s="8">
         <v>1</v>
@@ -10113,7 +10113,7 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="G69" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H69" s="8">
         <v>1</v>
@@ -10187,19 +10187,19 @@
       </c>
       <c r="Z69" s="11">
         <f>Y69*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B69)</f>
-        <v>1760.8959106694499</v>
+        <v>1760.8959106694797</v>
       </c>
       <c r="AA69" s="11">
         <f t="shared" ref="AA69:AA132" si="29">Z69*J69</f>
-        <v>1760.8959106694499</v>
+        <v>1760.8959106694797</v>
       </c>
       <c r="AB69" s="11">
         <f t="shared" ref="AB69:AB132" si="30">IF(AA69&lt;=0,0,(rate_below/100)*MIN(AA69,MAX(0,ceiling-D69))+(rate_above/100)*(AA69-MIN(AA69,MAX(0,ceiling-D69))))</f>
-        <v>554.68221186087669</v>
+        <v>554.68221186088613</v>
       </c>
       <c r="AC69" s="11">
         <f t="shared" ref="AC69:AC132" si="31">AA69+AB69</f>
-        <v>2315.5781225303267</v>
+        <v>2315.5781225303658</v>
       </c>
       <c r="AD69" s="12">
         <f t="shared" ref="AD69:AD132" si="32">SUMPRODUCT(($B$5:$B$216=B69)*($M$5:$M$216&lt;M69))+SUMPRODUCT(($B$5:$B$216=B69)*($M$5:$M$216=M69)*(ROW($M$5:$M$216)&lt;ROW(M69)))+1</f>
@@ -10238,7 +10238,7 @@
         <v>1.7</v>
       </c>
       <c r="G70" s="8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H70" s="8">
         <v>1</v>
@@ -10312,19 +10312,19 @@
       </c>
       <c r="Z70" s="11">
         <f>Y70*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B70)</f>
-        <v>1050.0256241220629</v>
+        <v>1050.0256241220804</v>
       </c>
       <c r="AA70" s="11">
         <f t="shared" si="29"/>
-        <v>1050.0256241220629</v>
+        <v>1050.0256241220804</v>
       </c>
       <c r="AB70" s="11">
         <f t="shared" si="30"/>
-        <v>330.75807159844982</v>
+        <v>330.75807159845533</v>
       </c>
       <c r="AC70" s="11">
         <f t="shared" si="31"/>
-        <v>1380.7836957205127</v>
+        <v>1380.7836957205359</v>
       </c>
       <c r="AD70" s="12">
         <f t="shared" si="32"/>
@@ -10363,7 +10363,7 @@
         <v>6.7</v>
       </c>
       <c r="G71" s="8">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H71" s="8">
         <v>1</v>
@@ -10488,7 +10488,7 @@
         <v>8.1</v>
       </c>
       <c r="G72" s="8">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H72" s="8">
         <v>1</v>
@@ -10613,7 +10613,7 @@
         <v>3.3</v>
       </c>
       <c r="G73" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H73" s="8">
         <v>1</v>
@@ -10687,19 +10687,19 @@
       </c>
       <c r="Z73" s="11">
         <f>Y73*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B73)</f>
-        <v>1845.7462065763477</v>
+        <v>1845.7462065763789</v>
       </c>
       <c r="AA73" s="11">
         <f t="shared" si="29"/>
-        <v>1845.7462065763477</v>
+        <v>1845.7462065763789</v>
       </c>
       <c r="AB73" s="11">
         <f t="shared" si="30"/>
-        <v>581.41005507154955</v>
+        <v>581.41005507155933</v>
       </c>
       <c r="AC73" s="11">
         <f t="shared" si="31"/>
-        <v>2427.1562616478973</v>
+        <v>2427.1562616479382</v>
       </c>
       <c r="AD73" s="12">
         <f t="shared" si="32"/>
@@ -10738,7 +10738,7 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="G74" s="8">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H74" s="8">
         <v>1</v>
@@ -10863,7 +10863,7 @@
         <v>3.9</v>
       </c>
       <c r="G75" s="8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H75" s="8">
         <v>1</v>
@@ -10937,19 +10937,19 @@
       </c>
       <c r="Z75" s="11">
         <f>Y75*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B75)</f>
-        <v>282.80091203786662</v>
+        <v>282.8009120378714</v>
       </c>
       <c r="AA75" s="11">
         <f t="shared" si="29"/>
-        <v>282.80091203786662</v>
+        <v>282.8009120378714</v>
       </c>
       <c r="AB75" s="11">
         <f t="shared" si="30"/>
-        <v>89.082287291927983</v>
+        <v>89.082287291929489</v>
       </c>
       <c r="AC75" s="11">
         <f t="shared" si="31"/>
-        <v>371.88319932979459</v>
+        <v>371.8831993298009</v>
       </c>
       <c r="AD75" s="12">
         <f t="shared" si="32"/>
@@ -10988,7 +10988,7 @@
         <v>6.6</v>
       </c>
       <c r="G76" s="8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H76" s="8">
         <v>1</v>
@@ -11062,19 +11062,19 @@
       </c>
       <c r="Z76" s="11">
         <f>Y76*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B76)</f>
-        <v>257.00506521754465</v>
+        <v>257.00506521754897</v>
       </c>
       <c r="AA76" s="11">
         <f t="shared" si="29"/>
-        <v>257.00506521754465</v>
+        <v>257.00506521754897</v>
       </c>
       <c r="AB76" s="11">
         <f t="shared" si="30"/>
-        <v>80.956595543526561</v>
+        <v>80.956595543527925</v>
       </c>
       <c r="AC76" s="11">
         <f t="shared" si="31"/>
-        <v>337.96166076107124</v>
+        <v>337.96166076107693</v>
       </c>
       <c r="AD76" s="12">
         <f t="shared" si="32"/>
@@ -11113,7 +11113,7 @@
         <v>8.9</v>
       </c>
       <c r="G77" s="8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H77" s="8">
         <v>1</v>
@@ -11238,7 +11238,7 @@
         <v>5.5</v>
       </c>
       <c r="G78" s="8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H78" s="8">
         <v>1</v>
@@ -11312,19 +11312,19 @@
       </c>
       <c r="Z78" s="11">
         <f>Y78*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B78)</f>
-        <v>1437.8541971413017</v>
+        <v>1437.854197141326</v>
       </c>
       <c r="AA78" s="11">
         <f t="shared" si="29"/>
-        <v>1437.8541971413017</v>
+        <v>1437.854197141326</v>
       </c>
       <c r="AB78" s="11">
         <f t="shared" si="30"/>
-        <v>452.92407209951006</v>
+        <v>452.92407209951773</v>
       </c>
       <c r="AC78" s="11">
         <f t="shared" si="31"/>
-        <v>1890.7782692408118</v>
+        <v>1890.7782692408437</v>
       </c>
       <c r="AD78" s="12">
         <f t="shared" si="32"/>
@@ -11363,7 +11363,7 @@
         <v>3.3</v>
       </c>
       <c r="G79" s="8">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H79" s="8">
         <v>1</v>
@@ -11488,7 +11488,7 @@
         <v>5.8</v>
       </c>
       <c r="G80" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H80" s="8">
         <v>1</v>
@@ -11613,7 +11613,7 @@
         <v>2.9</v>
       </c>
       <c r="G81" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H81" s="8">
         <v>1</v>
@@ -11687,19 +11687,19 @@
       </c>
       <c r="Z81" s="11">
         <f>Y81*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B81)</f>
-        <v>1989.4659245752916</v>
+        <v>1989.4659245753251</v>
       </c>
       <c r="AA81" s="11">
         <f t="shared" si="29"/>
-        <v>1989.4659245752916</v>
+        <v>1989.4659245753251</v>
       </c>
       <c r="AB81" s="11">
         <f t="shared" si="30"/>
-        <v>626.68176624121691</v>
+        <v>626.68176624122736</v>
       </c>
       <c r="AC81" s="11">
         <f t="shared" si="31"/>
-        <v>2616.1476908165087</v>
+        <v>2616.1476908165523</v>
       </c>
       <c r="AD81" s="12">
         <f t="shared" si="32"/>
@@ -11738,7 +11738,7 @@
         <v>7.5</v>
       </c>
       <c r="G82" s="8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H82" s="8">
         <v>1</v>
@@ -11863,7 +11863,7 @@
         <v>5.6</v>
       </c>
       <c r="G83" s="8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H83" s="8">
         <v>1</v>
@@ -11988,7 +11988,7 @@
         <v>10</v>
       </c>
       <c r="G84" s="8">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H84" s="8">
         <v>1</v>
@@ -12113,7 +12113,7 @@
         <v>6.4</v>
       </c>
       <c r="G85" s="8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H85" s="8">
         <v>1</v>
@@ -12238,7 +12238,7 @@
         <v>8.3000000000000007</v>
       </c>
       <c r="G86" s="8">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H86" s="8">
         <v>1</v>
@@ -12363,7 +12363,7 @@
         <v>6.1</v>
       </c>
       <c r="G87" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H87" s="8">
         <v>1</v>
@@ -12409,19 +12409,19 @@
       </c>
       <c r="S87" s="11">
         <f>R87*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B87)</f>
-        <v>2708.3538702662081</v>
+        <v>2708.3538702661713</v>
       </c>
       <c r="T87" s="11">
         <f t="shared" si="25"/>
-        <v>2708.3538702662081</v>
+        <v>2708.3538702661713</v>
       </c>
       <c r="U87" s="11">
         <f t="shared" si="26"/>
-        <v>26.000197154555597</v>
+        <v>26.000197154555241</v>
       </c>
       <c r="V87" s="11">
         <f t="shared" si="27"/>
-        <v>2734.3540674207638</v>
+        <v>2734.3540674207266</v>
       </c>
       <c r="W87" s="12">
         <f>IF(AND(C87="F",M87&lt;O87,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B87)=1),1,0)</f>
@@ -12437,19 +12437,19 @@
       </c>
       <c r="Z87" s="11">
         <f>Y87*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B87)</f>
-        <v>11393.879179732585</v>
+        <v>11393.879179732548</v>
       </c>
       <c r="AA87" s="11">
         <f t="shared" si="29"/>
-        <v>11393.879179732585</v>
+        <v>11393.879179732548</v>
       </c>
       <c r="AB87" s="11">
         <f t="shared" si="30"/>
-        <v>109.38124012543281</v>
+        <v>109.38124012543246</v>
       </c>
       <c r="AC87" s="11">
         <f t="shared" si="31"/>
-        <v>11503.260419858017</v>
+        <v>11503.260419857981</v>
       </c>
       <c r="AD87" s="12">
         <f t="shared" si="32"/>
@@ -12488,7 +12488,7 @@
         <v>7.1</v>
       </c>
       <c r="G88" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H88" s="8">
         <v>1</v>
@@ -12534,19 +12534,19 @@
       </c>
       <c r="S88" s="11">
         <f>R88*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B88)</f>
-        <v>1233.50232813094</v>
+        <v>1233.5023281309232</v>
       </c>
       <c r="T88" s="11">
         <f t="shared" si="25"/>
-        <v>1233.50232813094</v>
+        <v>1233.5023281309232</v>
       </c>
       <c r="U88" s="11">
         <f t="shared" si="26"/>
-        <v>11.841622350057023</v>
+        <v>11.841622350056861</v>
       </c>
       <c r="V88" s="11">
         <f t="shared" si="27"/>
-        <v>1245.3439504809969</v>
+        <v>1245.3439504809801</v>
       </c>
       <c r="W88" s="12">
         <f>IF(AND(C88="F",M88&lt;O88,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B88)=1),1,0)</f>
@@ -12562,19 +12562,19 @@
       </c>
       <c r="Z88" s="11">
         <f>Y88*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B88)</f>
-        <v>5189.2688946372291</v>
+        <v>5189.2688946372118</v>
       </c>
       <c r="AA88" s="11">
         <f t="shared" si="29"/>
-        <v>5189.2688946372291</v>
+        <v>5189.2688946372118</v>
       </c>
       <c r="AB88" s="11">
         <f t="shared" si="30"/>
-        <v>49.816981388517398</v>
+        <v>49.816981388517227</v>
       </c>
       <c r="AC88" s="11">
         <f t="shared" si="31"/>
-        <v>5239.0858760257461</v>
+        <v>5239.0858760257288</v>
       </c>
       <c r="AD88" s="12">
         <f t="shared" si="32"/>
@@ -12613,7 +12613,7 @@
         <v>8.1</v>
       </c>
       <c r="G89" s="8">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H89" s="8">
         <v>1</v>
@@ -12738,7 +12738,7 @@
         <v>5.9</v>
       </c>
       <c r="G90" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H90" s="8">
         <v>1</v>
@@ -12863,7 +12863,7 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="G91" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H91" s="8">
         <v>1</v>
@@ -12909,19 +12909,19 @@
       </c>
       <c r="S91" s="11">
         <f>R91*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B91)</f>
-        <v>405.03984494479784</v>
+        <v>405.03984494479232</v>
       </c>
       <c r="T91" s="11">
         <f t="shared" si="25"/>
-        <v>405.03984494479784</v>
+        <v>405.03984494479232</v>
       </c>
       <c r="U91" s="11">
         <f t="shared" si="26"/>
-        <v>3.8883825114700588</v>
+        <v>3.8883825114700059</v>
       </c>
       <c r="V91" s="11">
         <f t="shared" si="27"/>
-        <v>408.9282274562679</v>
+        <v>408.92822745626233</v>
       </c>
       <c r="W91" s="12">
         <f>IF(AND(C91="F",M91&lt;O91,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B91)=1),1,0)</f>
@@ -12937,19 +12937,19 @@
       </c>
       <c r="Z91" s="11">
         <f>Y91*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B91)</f>
-        <v>1703.9778689721343</v>
+        <v>1703.9778689721288</v>
       </c>
       <c r="AA91" s="11">
         <f t="shared" si="29"/>
-        <v>1703.9778689721343</v>
+        <v>1703.9778689721288</v>
       </c>
       <c r="AB91" s="11">
         <f t="shared" si="30"/>
-        <v>16.358187542132487</v>
+        <v>16.358187542132434</v>
       </c>
       <c r="AC91" s="11">
         <f t="shared" si="31"/>
-        <v>1720.3360565142668</v>
+        <v>1720.3360565142611</v>
       </c>
       <c r="AD91" s="12">
         <f t="shared" si="32"/>
@@ -12988,7 +12988,7 @@
         <v>8.8000000000000007</v>
       </c>
       <c r="G92" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H92" s="8">
         <v>1</v>
@@ -13113,7 +13113,7 @@
         <v>1.3</v>
       </c>
       <c r="G93" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H93" s="8">
         <v>1</v>
@@ -13238,7 +13238,7 @@
         <v>2.7</v>
       </c>
       <c r="G94" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H94" s="8">
         <v>1</v>
@@ -13363,7 +13363,7 @@
         <v>8.3000000000000007</v>
       </c>
       <c r="G95" s="8">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H95" s="8">
         <v>1</v>
@@ -13488,7 +13488,7 @@
         <v>10.7</v>
       </c>
       <c r="G96" s="8">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H96" s="8">
         <v>1</v>
@@ -13613,7 +13613,7 @@
         <v>8.9</v>
       </c>
       <c r="G97" s="8">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H97" s="8">
         <v>1</v>
@@ -13738,7 +13738,7 @@
         <v>9.9</v>
       </c>
       <c r="G98" s="8">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H98" s="8">
         <v>1</v>
@@ -13863,7 +13863,7 @@
         <v>4.8</v>
       </c>
       <c r="G99" s="8">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H99" s="8">
         <v>1</v>
@@ -13988,7 +13988,7 @@
         <v>13</v>
       </c>
       <c r="G100" s="8">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H100" s="8">
         <v>1</v>
@@ -14113,7 +14113,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="G101" s="8">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H101" s="8">
         <v>1</v>
@@ -14238,7 +14238,7 @@
         <v>8.4</v>
       </c>
       <c r="G102" s="8">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H102" s="8">
         <v>1</v>
@@ -14363,7 +14363,7 @@
         <v>8.1</v>
       </c>
       <c r="G103" s="8">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H103" s="8">
         <v>1</v>
@@ -14488,7 +14488,7 @@
         <v>12.9</v>
       </c>
       <c r="G104" s="8">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H104" s="8">
         <v>1</v>
@@ -14613,7 +14613,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="G105" s="8">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H105" s="8">
         <v>1</v>
@@ -14738,7 +14738,7 @@
         <v>7</v>
       </c>
       <c r="G106" s="8">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H106" s="8">
         <v>1</v>
@@ -14863,7 +14863,7 @@
         <v>5.9</v>
       </c>
       <c r="G107" s="8">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H107" s="8">
         <v>1</v>
@@ -14988,7 +14988,7 @@
         <v>5.5</v>
       </c>
       <c r="G108" s="8">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H108" s="8">
         <v>1</v>
@@ -15113,7 +15113,7 @@
         <v>8.9</v>
       </c>
       <c r="G109" s="8">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H109" s="8">
         <v>1</v>
@@ -15238,7 +15238,7 @@
         <v>12.1</v>
       </c>
       <c r="G110" s="8">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H110" s="8">
         <v>1</v>
@@ -15363,7 +15363,7 @@
         <v>7.9</v>
       </c>
       <c r="G111" s="8">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H111" s="8">
         <v>1</v>
@@ -15488,7 +15488,7 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="G112" s="8">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H112" s="8">
         <v>1</v>
@@ -15613,7 +15613,7 @@
         <v>5.5</v>
       </c>
       <c r="G113" s="8">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H113" s="8">
         <v>1</v>
@@ -15738,7 +15738,7 @@
         <v>7</v>
       </c>
       <c r="G114" s="8">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H114" s="8">
         <v>1</v>
@@ -15863,7 +15863,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="G115" s="8">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H115" s="8">
         <v>1</v>
@@ -15988,7 +15988,7 @@
         <v>4.9000000000000004</v>
       </c>
       <c r="G116" s="8">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H116" s="8">
         <v>1</v>
@@ -16113,7 +16113,7 @@
         <v>5.9</v>
       </c>
       <c r="G117" s="8">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H117" s="8">
         <v>1</v>
@@ -16238,7 +16238,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="G118" s="8">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H118" s="8">
         <v>1</v>
@@ -16363,7 +16363,7 @@
         <v>5.9</v>
       </c>
       <c r="G119" s="8">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H119" s="8">
         <v>1</v>
@@ -16488,7 +16488,7 @@
         <v>11.9</v>
       </c>
       <c r="G120" s="8">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H120" s="8">
         <v>1</v>
@@ -16613,7 +16613,7 @@
         <v>12.4</v>
       </c>
       <c r="G121" s="8">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H121" s="8">
         <v>1</v>
@@ -16738,7 +16738,7 @@
         <v>11.3</v>
       </c>
       <c r="G122" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H122" s="8">
         <v>0.5</v>
@@ -16863,7 +16863,7 @@
         <v>15.7</v>
       </c>
       <c r="G123" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H123" s="8">
         <v>1</v>
@@ -16988,7 +16988,7 @@
         <v>10.6</v>
       </c>
       <c r="G124" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H124" s="8">
         <v>1</v>
@@ -17113,7 +17113,7 @@
         <v>8</v>
       </c>
       <c r="G125" s="8">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H125" s="8">
         <v>1</v>
@@ -17238,7 +17238,7 @@
         <v>3.6</v>
       </c>
       <c r="G126" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H126" s="8">
         <v>1</v>
@@ -17363,7 +17363,7 @@
         <v>7.8</v>
       </c>
       <c r="G127" s="8">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H127" s="8">
         <v>1</v>
@@ -17409,19 +17409,19 @@
       </c>
       <c r="S127" s="11">
         <f>R127*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B127)</f>
-        <v>797.33167942695923</v>
+        <v>797.33167942697287</v>
       </c>
       <c r="T127" s="11">
         <f t="shared" si="25"/>
-        <v>797.33167942695923</v>
+        <v>797.33167942697287</v>
       </c>
       <c r="U127" s="11">
         <f t="shared" si="26"/>
-        <v>251.15947901949215</v>
+        <v>251.15947901949644</v>
       </c>
       <c r="V127" s="11">
         <f t="shared" si="27"/>
-        <v>1048.4911584464514</v>
+        <v>1048.4911584464694</v>
       </c>
       <c r="W127" s="12">
         <f>IF(AND(C127="F",M127&lt;O127,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B127)=1),1,0)</f>
@@ -17437,19 +17437,19 @@
       </c>
       <c r="Z127" s="11">
         <f>Y127*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B127)</f>
-        <v>3200.0171770132965</v>
+        <v>3200.0171770133102</v>
       </c>
       <c r="AA127" s="11">
         <f t="shared" si="29"/>
-        <v>3200.0171770132965</v>
+        <v>3200.0171770133102</v>
       </c>
       <c r="AB127" s="11">
         <f t="shared" si="30"/>
-        <v>1008.0054107591884</v>
+        <v>1008.0054107591927</v>
       </c>
       <c r="AC127" s="11">
         <f t="shared" si="31"/>
-        <v>4208.0225877724852</v>
+        <v>4208.0225877725024</v>
       </c>
       <c r="AD127" s="12">
         <f t="shared" si="32"/>
@@ -17488,7 +17488,7 @@
         <v>7.4</v>
       </c>
       <c r="G128" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H128" s="8">
         <v>1</v>
@@ -17534,19 +17534,19 @@
       </c>
       <c r="S128" s="11">
         <f>R128*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B128)</f>
-        <v>1480.8226870800268</v>
+        <v>1480.8226870800522</v>
       </c>
       <c r="T128" s="11">
         <f t="shared" si="25"/>
-        <v>1480.8226870800268</v>
+        <v>1480.8226870800522</v>
       </c>
       <c r="U128" s="11">
         <f t="shared" si="26"/>
-        <v>466.45914643020842</v>
+        <v>466.45914643021644</v>
       </c>
       <c r="V128" s="11">
         <f t="shared" si="27"/>
-        <v>1947.2818335102352</v>
+        <v>1947.2818335102686</v>
       </c>
       <c r="W128" s="12">
         <f>IF(AND(C128="F",M128&lt;O128,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B128)=1),1,0)</f>
@@ -17562,19 +17562,19 @@
       </c>
       <c r="Z128" s="11">
         <f>Y128*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B128)</f>
-        <v>5943.1453145982314</v>
+        <v>5943.1453145982559</v>
       </c>
       <c r="AA128" s="11">
         <f t="shared" si="29"/>
-        <v>5943.1453145982314</v>
+        <v>5943.1453145982559</v>
       </c>
       <c r="AB128" s="11">
         <f t="shared" si="30"/>
-        <v>1872.0907740984428</v>
+        <v>1872.0907740984505</v>
       </c>
       <c r="AC128" s="11">
         <f t="shared" si="31"/>
-        <v>7815.2360886966744</v>
+        <v>7815.2360886967062</v>
       </c>
       <c r="AD128" s="12">
         <f t="shared" si="32"/>
@@ -17613,7 +17613,7 @@
         <v>5.9</v>
       </c>
       <c r="G129" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H129" s="8">
         <v>1</v>
@@ -17659,19 +17659,19 @@
       </c>
       <c r="S129" s="11">
         <f>R129*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B129)</f>
-        <v>911.94727329922046</v>
+        <v>911.94727329923614</v>
       </c>
       <c r="T129" s="11">
         <f t="shared" si="25"/>
-        <v>911.94727329922046</v>
+        <v>911.94727329923614</v>
       </c>
       <c r="U129" s="11">
         <f t="shared" si="26"/>
-        <v>287.26339108925447</v>
+        <v>287.26339108925941</v>
       </c>
       <c r="V129" s="11">
         <f t="shared" si="27"/>
-        <v>1199.2106643884749</v>
+        <v>1199.2106643884956</v>
       </c>
       <c r="W129" s="12">
         <f>IF(AND(C129="F",M129&lt;O129,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B129)=1),1,0)</f>
@@ -17687,19 +17687,19 @@
       </c>
       <c r="Z129" s="11">
         <f>Y129*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B129)</f>
-        <v>3660.016294831385</v>
+        <v>3660.0162948314005</v>
       </c>
       <c r="AA129" s="11">
         <f t="shared" si="29"/>
-        <v>3660.016294831385</v>
+        <v>3660.0162948314005</v>
       </c>
       <c r="AB129" s="11">
         <f t="shared" si="30"/>
-        <v>1152.9051328718863</v>
+        <v>1152.9051328718911</v>
       </c>
       <c r="AC129" s="11">
         <f t="shared" si="31"/>
-        <v>4812.9214277032715</v>
+        <v>4812.9214277032916</v>
       </c>
       <c r="AD129" s="12">
         <f t="shared" si="32"/>
@@ -17738,7 +17738,7 @@
         <v>11.8</v>
       </c>
       <c r="G130" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H130" s="8">
         <v>1</v>
@@ -17863,7 +17863,7 @@
         <v>18.5</v>
       </c>
       <c r="G131" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H131" s="8">
         <v>1</v>
@@ -17988,7 +17988,7 @@
         <v>7.1</v>
       </c>
       <c r="G132" s="8">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H132" s="8">
         <v>1</v>
@@ -18113,7 +18113,7 @@
         <v>3.4</v>
       </c>
       <c r="G133" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H133" s="8">
         <v>1</v>
@@ -18238,7 +18238,7 @@
         <v>6.8</v>
       </c>
       <c r="G134" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H134" s="8">
         <v>1</v>
@@ -18284,19 +18284,19 @@
       </c>
       <c r="S134" s="11">
         <f>R134*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B134)</f>
-        <v>1130.5951467013344</v>
+        <v>1130.5951467013538</v>
       </c>
       <c r="T134" s="11">
         <f t="shared" si="43"/>
-        <v>1130.5951467013344</v>
+        <v>1130.5951467013538</v>
       </c>
       <c r="U134" s="11">
         <f t="shared" si="44"/>
-        <v>356.13747121092035</v>
+        <v>356.13747121092644</v>
       </c>
       <c r="V134" s="11">
         <f t="shared" si="45"/>
-        <v>1486.7326179122547</v>
+        <v>1486.7326179122801</v>
       </c>
       <c r="W134" s="12">
         <f>IF(AND(C134="F",M134&lt;O134,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B134)=1),1,0)</f>
@@ -18312,19 +18312,19 @@
       </c>
       <c r="Z134" s="11">
         <f>Y134*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B134)</f>
-        <v>4537.5393741941034</v>
+        <v>4537.5393741941225</v>
       </c>
       <c r="AA134" s="11">
         <f t="shared" si="47"/>
-        <v>4537.5393741941034</v>
+        <v>4537.5393741941225</v>
       </c>
       <c r="AB134" s="11">
         <f t="shared" si="48"/>
-        <v>1429.3249028711425</v>
+        <v>1429.3249028711487</v>
       </c>
       <c r="AC134" s="11">
         <f t="shared" si="49"/>
-        <v>5966.8642770652459</v>
+        <v>5966.8642770652714</v>
       </c>
       <c r="AD134" s="12">
         <f t="shared" si="50"/>
@@ -18363,7 +18363,7 @@
         <v>18.899999999999999</v>
       </c>
       <c r="G135" s="8">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H135" s="8">
         <v>1</v>
@@ -18488,7 +18488,7 @@
         <v>5.5</v>
       </c>
       <c r="G136" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H136" s="8">
         <v>1</v>
@@ -18534,19 +18534,19 @@
       </c>
       <c r="S136" s="11">
         <f>R136*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B136)</f>
-        <v>1644.3093868299982</v>
+        <v>1644.3093868300264</v>
       </c>
       <c r="T136" s="11">
         <f t="shared" si="43"/>
-        <v>1644.3093868299982</v>
+        <v>1644.3093868300264</v>
       </c>
       <c r="U136" s="11">
         <f t="shared" si="44"/>
-        <v>517.95745685144948</v>
+        <v>517.95745685145835</v>
       </c>
       <c r="V136" s="11">
         <f t="shared" si="45"/>
-        <v>2162.2668436814474</v>
+        <v>2162.2668436814847</v>
       </c>
       <c r="W136" s="12">
         <f>IF(AND(C136="F",M136&lt;O136,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B136)=1),1,0)</f>
@@ -18562,19 +18562,19 @@
       </c>
       <c r="Z136" s="11">
         <f>Y136*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B136)</f>
-        <v>6599.2841096717166</v>
+        <v>6599.2841096717448</v>
       </c>
       <c r="AA136" s="11">
         <f t="shared" si="47"/>
-        <v>6599.2841096717166</v>
+        <v>6599.2841096717448</v>
       </c>
       <c r="AB136" s="11">
         <f t="shared" si="48"/>
-        <v>2078.7744945465906</v>
+        <v>2078.7744945465997</v>
       </c>
       <c r="AC136" s="11">
         <f t="shared" si="49"/>
-        <v>8678.0586042183077</v>
+        <v>8678.058604218344</v>
       </c>
       <c r="AD136" s="12">
         <f t="shared" si="50"/>
@@ -18613,7 +18613,7 @@
         <v>6.2</v>
       </c>
       <c r="G137" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H137" s="8">
         <v>0.5</v>
@@ -18659,19 +18659,19 @@
       </c>
       <c r="S137" s="11">
         <f>R137*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B137)</f>
-        <v>1355.35656434868</v>
+        <v>1355.3565643487034</v>
       </c>
       <c r="T137" s="11">
         <f t="shared" si="43"/>
-        <v>677.67828217433998</v>
+        <v>677.67828217435169</v>
       </c>
       <c r="U137" s="11">
         <f t="shared" si="44"/>
-        <v>213.46865888491709</v>
+        <v>213.46865888492079</v>
       </c>
       <c r="V137" s="11">
         <f t="shared" si="45"/>
-        <v>891.14694105925707</v>
+        <v>891.14694105927242</v>
       </c>
       <c r="W137" s="12">
         <f>IF(AND(C137="F",M137&lt;O137,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B137)=1),1,0)</f>
@@ -18687,19 +18687,19 @@
       </c>
       <c r="Z137" s="11">
         <f>Y137*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B137)</f>
-        <v>5439.5985996826503</v>
+        <v>5439.5985996826739</v>
       </c>
       <c r="AA137" s="11">
         <f t="shared" si="47"/>
-        <v>2719.7992998413251</v>
+        <v>2719.799299841337</v>
       </c>
       <c r="AB137" s="11">
         <f t="shared" si="48"/>
-        <v>856.73677945001748</v>
+        <v>856.73677945002112</v>
       </c>
       <c r="AC137" s="11">
         <f t="shared" si="49"/>
-        <v>3576.5360792913425</v>
+        <v>3576.536079291358</v>
       </c>
       <c r="AD137" s="12">
         <f t="shared" si="50"/>
@@ -18738,7 +18738,7 @@
         <v>9.9</v>
       </c>
       <c r="G138" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H138" s="8">
         <v>1</v>
@@ -18784,19 +18784,19 @@
       </c>
       <c r="S138" s="11">
         <f>R138*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B138)</f>
-        <v>1184.5821959620084</v>
+        <v>1184.5821959620289</v>
       </c>
       <c r="T138" s="11">
         <f t="shared" si="43"/>
-        <v>1184.5821959620084</v>
+        <v>1184.5821959620289</v>
       </c>
       <c r="U138" s="11">
         <f t="shared" si="44"/>
-        <v>373.14339172803267</v>
+        <v>373.14339172803909</v>
       </c>
       <c r="V138" s="11">
         <f t="shared" si="45"/>
-        <v>1557.725587690041</v>
+        <v>1557.7255876900681</v>
       </c>
       <c r="W138" s="12">
         <f>IF(AND(C138="F",M138&lt;O138,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B138)=1),1,0)</f>
@@ -18812,19 +18812,19 @@
       </c>
       <c r="Z138" s="11">
         <f>Y138*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B138)</f>
-        <v>4754.211418498905</v>
+        <v>4754.211418498925</v>
       </c>
       <c r="AA138" s="11">
         <f t="shared" si="47"/>
-        <v>4754.211418498905</v>
+        <v>4754.211418498925</v>
       </c>
       <c r="AB138" s="11">
         <f t="shared" si="48"/>
-        <v>1497.5765968271551</v>
+        <v>1497.5765968271614</v>
       </c>
       <c r="AC138" s="11">
         <f t="shared" si="49"/>
-        <v>6251.7880153260603</v>
+        <v>6251.7880153260867</v>
       </c>
       <c r="AD138" s="12">
         <f t="shared" si="50"/>
@@ -18863,7 +18863,7 @@
         <v>15.1</v>
       </c>
       <c r="G139" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H139" s="8">
         <v>1</v>
@@ -18988,7 +18988,7 @@
         <v>14.9</v>
       </c>
       <c r="G140" s="8">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H140" s="8">
         <v>1</v>
@@ -19113,7 +19113,7 @@
         <v>13</v>
       </c>
       <c r="G141" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H141" s="8">
         <v>1</v>
@@ -19238,7 +19238,7 @@
         <v>12.1</v>
       </c>
       <c r="G142" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H142" s="8">
         <v>0.5</v>
@@ -19363,7 +19363,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="G143" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H143" s="8">
         <v>1</v>
@@ -19409,19 +19409,19 @@
       </c>
       <c r="S143" s="11">
         <f>R143*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B143)</f>
-        <v>1854.3804839876757</v>
+        <v>1854.3804839877077</v>
       </c>
       <c r="T143" s="11">
         <f t="shared" si="43"/>
-        <v>1854.3804839876757</v>
+        <v>1854.3804839877077</v>
       </c>
       <c r="U143" s="11">
         <f t="shared" si="44"/>
-        <v>584.12985245611787</v>
+        <v>584.12985245612799</v>
       </c>
       <c r="V143" s="11">
         <f t="shared" si="45"/>
-        <v>2438.5103364437937</v>
+        <v>2438.5103364438355</v>
       </c>
       <c r="W143" s="12">
         <f>IF(AND(C143="F",M143&lt;O143,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B143)=1),1,0)</f>
@@ -19437,19 +19437,19 @@
       </c>
       <c r="Z143" s="11">
         <f>Y143*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B143)</f>
-        <v>7442.3850884033391</v>
+        <v>7442.3850884033709</v>
       </c>
       <c r="AA143" s="11">
         <f t="shared" si="47"/>
-        <v>7442.3850884033391</v>
+        <v>7442.3850884033709</v>
       </c>
       <c r="AB143" s="11">
         <f t="shared" si="48"/>
-        <v>2344.351302847052</v>
+        <v>2344.351302847062</v>
       </c>
       <c r="AC143" s="11">
         <f t="shared" si="49"/>
-        <v>9786.7363912503915</v>
+        <v>9786.7363912504334</v>
       </c>
       <c r="AD143" s="12">
         <f t="shared" si="50"/>
@@ -19488,7 +19488,7 @@
         <v>4.2</v>
       </c>
       <c r="G144" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H144" s="8">
         <v>1</v>
@@ -19613,7 +19613,7 @@
         <v>13</v>
       </c>
       <c r="G145" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H145" s="8">
         <v>1</v>
@@ -19738,7 +19738,7 @@
         <v>8.1</v>
       </c>
       <c r="G146" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H146" s="8">
         <v>1</v>
@@ -19784,19 +19784,19 @@
       </c>
       <c r="S146" s="11">
         <f>R146*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B146)</f>
-        <v>2262.0478090789188</v>
+        <v>2262.0478090789579</v>
       </c>
       <c r="T146" s="11">
         <f t="shared" si="43"/>
-        <v>2262.0478090789188</v>
+        <v>2262.0478090789579</v>
       </c>
       <c r="U146" s="11">
         <f t="shared" si="44"/>
-        <v>712.54505985985941</v>
+        <v>712.5450598598718</v>
       </c>
       <c r="V146" s="11">
         <f t="shared" si="45"/>
-        <v>2974.5928689387783</v>
+        <v>2974.5928689388297</v>
       </c>
       <c r="W146" s="12">
         <f>IF(AND(C146="F",M146&lt;O146,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B146)=1),1,0)</f>
@@ -19812,19 +19812,19 @@
       </c>
       <c r="Z146" s="11">
         <f>Y146*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B146)</f>
-        <v>9078.5203084871737</v>
+        <v>9078.5203084872119</v>
       </c>
       <c r="AA146" s="11">
         <f t="shared" si="47"/>
-        <v>9078.5203084871737</v>
+        <v>9078.5203084872119</v>
       </c>
       <c r="AB146" s="11">
         <f t="shared" si="48"/>
-        <v>2859.7338971734598</v>
+        <v>2859.7338971734716</v>
       </c>
       <c r="AC146" s="11">
         <f t="shared" si="49"/>
-        <v>11938.254205660633</v>
+        <v>11938.254205660684</v>
       </c>
       <c r="AD146" s="12">
         <f t="shared" si="50"/>
@@ -19863,7 +19863,7 @@
         <v>11.4</v>
       </c>
       <c r="G147" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H147" s="8">
         <v>1</v>
@@ -19988,7 +19988,7 @@
         <v>11.5</v>
       </c>
       <c r="G148" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H148" s="8">
         <v>1</v>
@@ -20034,19 +20034,19 @@
       </c>
       <c r="S148" s="11">
         <f>R148*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B148)</f>
-        <v>811.24302911346024</v>
+        <v>811.24302911347422</v>
       </c>
       <c r="T148" s="11">
         <f t="shared" si="43"/>
-        <v>811.24302911346024</v>
+        <v>811.24302911347422</v>
       </c>
       <c r="U148" s="11">
         <f t="shared" si="44"/>
-        <v>255.54155417073997</v>
+        <v>255.54155417074438</v>
       </c>
       <c r="V148" s="11">
         <f t="shared" si="45"/>
-        <v>1066.7845832842002</v>
+        <v>1066.7845832842186</v>
       </c>
       <c r="W148" s="12">
         <f>IF(AND(C148="F",M148&lt;O148,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B148)=1),1,0)</f>
@@ -20062,19 +20062,19 @@
       </c>
       <c r="Z148" s="11">
         <f>Y148*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B148)</f>
-        <v>3255.8490962771039</v>
+        <v>3255.849096277118</v>
       </c>
       <c r="AA148" s="11">
         <f t="shared" si="47"/>
-        <v>3255.8490962771039</v>
+        <v>3255.849096277118</v>
       </c>
       <c r="AB148" s="11">
         <f t="shared" si="48"/>
-        <v>1025.5924653272878</v>
+        <v>1025.5924653272921</v>
       </c>
       <c r="AC148" s="11">
         <f t="shared" si="49"/>
-        <v>4281.4415616043916</v>
+        <v>4281.4415616044098</v>
       </c>
       <c r="AD148" s="12">
         <f t="shared" si="50"/>
@@ -20113,7 +20113,7 @@
         <v>18.399999999999999</v>
       </c>
       <c r="G149" s="8">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H149" s="8">
         <v>1</v>
@@ -20238,7 +20238,7 @@
         <v>15.6</v>
       </c>
       <c r="G150" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H150" s="8">
         <v>0.8</v>
@@ -20363,7 +20363,7 @@
         <v>5.5</v>
       </c>
       <c r="G151" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H151" s="8">
         <v>1</v>
@@ -20488,7 +20488,7 @@
         <v>18.600000000000001</v>
       </c>
       <c r="G152" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H152" s="8">
         <v>1</v>
@@ -20613,7 +20613,7 @@
         <v>12.8</v>
       </c>
       <c r="G153" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H153" s="8">
         <v>1</v>
@@ -20738,7 +20738,7 @@
         <v>7.8</v>
       </c>
       <c r="G154" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H154" s="8">
         <v>1</v>
@@ -20784,19 +20784,19 @@
       </c>
       <c r="S154" s="11">
         <f>R154*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B154)</f>
-        <v>1813.9161087528785</v>
+        <v>1813.9161087529096</v>
       </c>
       <c r="T154" s="11">
         <f t="shared" si="43"/>
-        <v>1813.9161087528785</v>
+        <v>1813.9161087529096</v>
       </c>
       <c r="U154" s="11">
         <f t="shared" si="44"/>
-        <v>571.38357425715674</v>
+        <v>571.38357425716652</v>
       </c>
       <c r="V154" s="11">
         <f t="shared" si="45"/>
-        <v>2385.2996830100351</v>
+        <v>2385.299683010076</v>
       </c>
       <c r="W154" s="12">
         <f>IF(AND(C154="F",M154&lt;O154,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B154)=1),1,0)</f>
@@ -20812,19 +20812,19 @@
       </c>
       <c r="Z154" s="11">
         <f>Y154*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B154)</f>
-        <v>7279.9850494364637</v>
+        <v>7279.9850494364937</v>
       </c>
       <c r="AA154" s="11">
         <f t="shared" si="47"/>
-        <v>7279.9850494364637</v>
+        <v>7279.9850494364937</v>
       </c>
       <c r="AB154" s="11">
         <f t="shared" si="48"/>
-        <v>2293.1952905724861</v>
+        <v>2293.1952905724957</v>
       </c>
       <c r="AC154" s="11">
         <f t="shared" si="49"/>
-        <v>9573.1803400089502</v>
+        <v>9573.1803400089884</v>
       </c>
       <c r="AD154" s="12">
         <f t="shared" si="50"/>
@@ -20863,7 +20863,7 @@
         <v>4.2</v>
       </c>
       <c r="G155" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H155" s="8">
         <v>1</v>
@@ -20988,7 +20988,7 @@
         <v>8.6999999999999993</v>
       </c>
       <c r="G156" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H156" s="8">
         <v>1</v>
@@ -21113,7 +21113,7 @@
         <v>12.4</v>
       </c>
       <c r="G157" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H157" s="8">
         <v>1</v>
@@ -21238,7 +21238,7 @@
         <v>9.6999999999999993</v>
       </c>
       <c r="G158" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H158" s="8">
         <v>1</v>
@@ -21363,7 +21363,7 @@
         <v>3.3</v>
       </c>
       <c r="G159" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H159" s="8">
         <v>1</v>
@@ -21409,19 +21409,19 @@
       </c>
       <c r="S159" s="11">
         <f>R159*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B159)</f>
-        <v>1870.0376351831471</v>
+        <v>1870.0376351831794</v>
       </c>
       <c r="T159" s="11">
         <f t="shared" si="43"/>
-        <v>1870.0376351831471</v>
+        <v>1870.0376351831794</v>
       </c>
       <c r="U159" s="11">
         <f t="shared" si="44"/>
-        <v>589.0618550826913</v>
+        <v>589.06185508270153</v>
       </c>
       <c r="V159" s="11">
         <f t="shared" si="45"/>
-        <v>2459.0994902658385</v>
+        <v>2459.0994902658808</v>
       </c>
       <c r="W159" s="12">
         <f>IF(AND(C159="F",M159&lt;O159,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B159)=1),1,0)</f>
@@ -21437,19 +21437,19 @@
       </c>
       <c r="Z159" s="11">
         <f>Y159*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B159)</f>
-        <v>7505.2236210508972</v>
+        <v>7505.2236210509291</v>
       </c>
       <c r="AA159" s="11">
         <f t="shared" si="47"/>
-        <v>7505.2236210508972</v>
+        <v>7505.2236210509291</v>
       </c>
       <c r="AB159" s="11">
         <f t="shared" si="48"/>
-        <v>2364.1454406310327</v>
+        <v>2364.1454406310427</v>
       </c>
       <c r="AC159" s="11">
         <f t="shared" si="49"/>
-        <v>9869.3690616819295</v>
+        <v>9869.3690616819713</v>
       </c>
       <c r="AD159" s="12">
         <f t="shared" si="50"/>
@@ -21488,7 +21488,7 @@
         <v>11.8</v>
       </c>
       <c r="G160" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H160" s="8">
         <v>1</v>
@@ -21613,7 +21613,7 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="G161" s="8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H161" s="8">
         <v>1</v>
@@ -21659,19 +21659,19 @@
       </c>
       <c r="S161" s="11">
         <f>R161*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B161)</f>
-        <v>865.27169351123496</v>
+        <v>865.27169351119778</v>
       </c>
       <c r="T161" s="11">
         <f t="shared" si="43"/>
-        <v>721.05974459269578</v>
+        <v>721.05974459266486</v>
       </c>
       <c r="U161" s="11">
         <f t="shared" si="44"/>
-        <v>227.13381954669916</v>
+        <v>227.13381954668944</v>
       </c>
       <c r="V161" s="11">
         <f t="shared" si="45"/>
-        <v>948.19356413939499</v>
+        <v>948.19356413935429</v>
       </c>
       <c r="W161" s="12">
         <f>IF(AND(C161="F",M161&lt;O161,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B161)=1),1,0)</f>
@@ -21687,19 +21687,19 @@
       </c>
       <c r="Z161" s="11">
         <f>Y161*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B161)</f>
-        <v>4475.5806085810009</v>
+        <v>4475.5806085809636</v>
       </c>
       <c r="AA161" s="11">
         <f t="shared" si="47"/>
-        <v>3729.6505071508341</v>
+        <v>3729.6505071508032</v>
       </c>
       <c r="AB161" s="11">
         <f t="shared" si="48"/>
-        <v>1174.8399097525128</v>
+        <v>1174.839909752503</v>
       </c>
       <c r="AC161" s="11">
         <f t="shared" si="49"/>
-        <v>4904.4904169033471</v>
+        <v>4904.4904169033061</v>
       </c>
       <c r="AD161" s="12">
         <f t="shared" si="50"/>
@@ -21738,7 +21738,7 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="G162" s="8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H162" s="8">
         <v>1</v>
@@ -21863,7 +21863,7 @@
         <v>6.1</v>
       </c>
       <c r="G163" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H163" s="8">
         <v>0.75</v>
@@ -21988,7 +21988,7 @@
         <v>12.6</v>
       </c>
       <c r="G164" s="8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H164" s="8">
         <v>1</v>
@@ -22113,7 +22113,7 @@
         <v>8.6</v>
       </c>
       <c r="G165" s="8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H165" s="8">
         <v>1</v>
@@ -22238,7 +22238,7 @@
         <v>4.3</v>
       </c>
       <c r="G166" s="8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H166" s="8">
         <v>1</v>
@@ -22284,19 +22284,19 @@
       </c>
       <c r="S166" s="11">
         <f>R166*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B166)</f>
-        <v>1022.3566300747239</v>
+        <v>1022.35663007468</v>
       </c>
       <c r="T166" s="11">
         <f t="shared" si="43"/>
-        <v>1022.3566300747239</v>
+        <v>1022.35663007468</v>
       </c>
       <c r="U166" s="11">
         <f t="shared" si="44"/>
-        <v>322.042338473538</v>
+        <v>322.04233847352418</v>
       </c>
       <c r="V166" s="11">
         <f t="shared" si="45"/>
-        <v>1344.3989685482618</v>
+        <v>1344.3989685482043</v>
       </c>
       <c r="W166" s="12">
         <f>IF(AND(C166="F",M166&lt;O166,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B166)=1),1,0)</f>
@@ -22312,19 +22312,19 @@
       </c>
       <c r="Z166" s="11">
         <f>Y166*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B166)</f>
-        <v>5288.0956847772377</v>
+        <v>5288.0956847771931</v>
       </c>
       <c r="AA166" s="11">
         <f t="shared" si="47"/>
-        <v>5288.0956847772377</v>
+        <v>5288.0956847771931</v>
       </c>
       <c r="AB166" s="11">
         <f t="shared" si="48"/>
-        <v>1665.7501407048298</v>
+        <v>1665.7501407048157</v>
       </c>
       <c r="AC166" s="11">
         <f t="shared" si="49"/>
-        <v>6953.8458254820671</v>
+        <v>6953.8458254820089</v>
       </c>
       <c r="AD166" s="12">
         <f t="shared" si="50"/>
@@ -22363,7 +22363,7 @@
         <v>8.9</v>
       </c>
       <c r="G167" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H167" s="8">
         <v>0.5</v>
@@ -22488,7 +22488,7 @@
         <v>1.4</v>
       </c>
       <c r="G168" s="8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H168" s="8">
         <v>1</v>
@@ -22613,7 +22613,7 @@
         <v>6.2</v>
       </c>
       <c r="G169" s="8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H169" s="8">
         <v>1</v>
@@ -22659,19 +22659,19 @@
       </c>
       <c r="S169" s="11">
         <f>R169*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B169)</f>
-        <v>570.50697137956786</v>
+        <v>570.5069713795433</v>
       </c>
       <c r="T169" s="11">
         <f t="shared" si="43"/>
-        <v>570.50697137956786</v>
+        <v>570.5069713795433</v>
       </c>
       <c r="U169" s="11">
         <f t="shared" si="44"/>
-        <v>179.70969598456387</v>
+        <v>179.70969598455613</v>
       </c>
       <c r="V169" s="11">
         <f t="shared" si="45"/>
-        <v>750.21666736413169</v>
+        <v>750.21666736409941</v>
       </c>
       <c r="W169" s="12">
         <f>IF(AND(C169="F",M169&lt;O169,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B169)=1),1,0)</f>
@@ -22687,19 +22687,19 @@
       </c>
       <c r="Z169" s="11">
         <f>Y169*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B169)</f>
-        <v>2950.9227648546862</v>
+        <v>2950.9227648546612</v>
       </c>
       <c r="AA169" s="11">
         <f t="shared" si="47"/>
-        <v>2950.9227648546862</v>
+        <v>2950.9227648546612</v>
       </c>
       <c r="AB169" s="11">
         <f t="shared" si="48"/>
-        <v>929.54067092922617</v>
+        <v>929.54067092921832</v>
       </c>
       <c r="AC169" s="11">
         <f t="shared" si="49"/>
-        <v>3880.4634357839122</v>
+        <v>3880.4634357838795</v>
       </c>
       <c r="AD169" s="12">
         <f t="shared" si="50"/>
@@ -22738,7 +22738,7 @@
         <v>14</v>
       </c>
       <c r="G170" s="8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H170" s="8">
         <v>1</v>
@@ -22863,7 +22863,7 @@
         <v>8.9</v>
       </c>
       <c r="G171" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H171" s="8">
         <v>1</v>
@@ -22988,7 +22988,7 @@
         <v>7.8</v>
       </c>
       <c r="G172" s="8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H172" s="8">
         <v>1</v>
@@ -23113,7 +23113,7 @@
         <v>5.3</v>
       </c>
       <c r="G173" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H173" s="8">
         <v>1</v>
@@ -23159,19 +23159,19 @@
       </c>
       <c r="S173" s="11">
         <f>R173*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B173)</f>
-        <v>729.48031537019756</v>
+        <v>729.48031537016618</v>
       </c>
       <c r="T173" s="11">
         <f t="shared" si="43"/>
-        <v>729.48031537019756</v>
+        <v>729.48031537016618</v>
       </c>
       <c r="U173" s="11">
         <f t="shared" si="44"/>
-        <v>229.78629934161222</v>
+        <v>229.78629934160236</v>
       </c>
       <c r="V173" s="11">
         <f t="shared" si="45"/>
-        <v>959.26661471180978</v>
+        <v>959.26661471176851</v>
       </c>
       <c r="W173" s="12">
         <f>IF(AND(C173="F",M173&lt;O173,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B173)=1),1,0)</f>
@@ -23187,19 +23187,19 @@
       </c>
       <c r="Z173" s="11">
         <f>Y173*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B173)</f>
-        <v>3773.2055472238994</v>
+        <v>3773.2055472238676</v>
       </c>
       <c r="AA173" s="11">
         <f t="shared" si="47"/>
-        <v>3773.2055472238994</v>
+        <v>3773.2055472238676</v>
       </c>
       <c r="AB173" s="11">
         <f t="shared" si="48"/>
-        <v>1188.5597473755283</v>
+        <v>1188.5597473755183</v>
       </c>
       <c r="AC173" s="11">
         <f t="shared" si="49"/>
-        <v>4961.7652945994278</v>
+        <v>4961.7652945993859</v>
       </c>
       <c r="AD173" s="12">
         <f t="shared" si="50"/>
@@ -23238,7 +23238,7 @@
         <v>3</v>
       </c>
       <c r="G174" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H174" s="8">
         <v>0.5</v>
@@ -23284,19 +23284,19 @@
       </c>
       <c r="S174" s="11">
         <f>R174*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B174)</f>
-        <v>327.27570619282392</v>
+        <v>327.27570619280988</v>
       </c>
       <c r="T174" s="11">
         <f t="shared" si="43"/>
-        <v>163.63785309641196</v>
+        <v>163.63785309640494</v>
       </c>
       <c r="U174" s="11">
         <f t="shared" si="44"/>
-        <v>51.545923725369768</v>
+        <v>51.545923725367558</v>
       </c>
       <c r="V174" s="11">
         <f t="shared" si="45"/>
-        <v>215.18377682178172</v>
+        <v>215.18377682177248</v>
       </c>
       <c r="W174" s="12">
         <f>IF(AND(C174="F",M174&lt;O174,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B174)=1),1,0)</f>
@@ -23312,19 +23312,19 @@
       </c>
       <c r="Z174" s="11">
         <f>Y174*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B174)</f>
-        <v>1692.8195100805494</v>
+        <v>1692.8195100805351</v>
       </c>
       <c r="AA174" s="11">
         <f t="shared" si="47"/>
-        <v>846.40975504027472</v>
+        <v>846.40975504026756</v>
       </c>
       <c r="AB174" s="11">
         <f t="shared" si="48"/>
-        <v>266.61907283768653</v>
+        <v>266.61907283768426</v>
       </c>
       <c r="AC174" s="11">
         <f t="shared" si="49"/>
-        <v>1113.0288278779612</v>
+        <v>1113.0288278779517</v>
       </c>
       <c r="AD174" s="12">
         <f t="shared" si="50"/>
@@ -23363,7 +23363,7 @@
         <v>5.4</v>
       </c>
       <c r="G175" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H175" s="8">
         <v>0.6</v>
@@ -23488,7 +23488,7 @@
         <v>6.9</v>
       </c>
       <c r="G176" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H176" s="8">
         <v>1</v>
@@ -23613,7 +23613,7 @@
         <v>3.5</v>
       </c>
       <c r="G177" s="8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H177" s="8">
         <v>1</v>
@@ -23659,19 +23659,19 @@
       </c>
       <c r="S177" s="11">
         <f>R177*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B177)</f>
-        <v>802.46806876301048</v>
+        <v>802.46806876297603</v>
       </c>
       <c r="T177" s="11">
         <f t="shared" si="43"/>
-        <v>802.46806876301048</v>
+        <v>802.46806876297603</v>
       </c>
       <c r="U177" s="11">
         <f t="shared" si="44"/>
-        <v>252.7774416603483</v>
+        <v>252.77744166033744</v>
       </c>
       <c r="V177" s="11">
         <f t="shared" si="45"/>
-        <v>1055.2455104233588</v>
+        <v>1055.2455104233136</v>
       </c>
       <c r="W177" s="12">
         <f>IF(AND(C177="F",M177&lt;O177,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B177)=1),1,0)</f>
@@ -23687,19 +23687,19 @@
       </c>
       <c r="Z177" s="11">
         <f>Y177*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B177)</f>
-        <v>4150.7315615364487</v>
+        <v>4150.7315615364132</v>
       </c>
       <c r="AA177" s="11">
         <f t="shared" si="47"/>
-        <v>4150.7315615364487</v>
+        <v>4150.7315615364132</v>
       </c>
       <c r="AB177" s="11">
         <f t="shared" si="48"/>
-        <v>1307.4804418839813</v>
+        <v>1307.4804418839701</v>
       </c>
       <c r="AC177" s="11">
         <f t="shared" si="49"/>
-        <v>5458.2120034204299</v>
+        <v>5458.2120034203836</v>
       </c>
       <c r="AD177" s="12">
         <f t="shared" si="50"/>
@@ -23738,7 +23738,7 @@
         <v>6.2</v>
       </c>
       <c r="G178" s="8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H178" s="8">
         <v>1</v>
@@ -23784,19 +23784,19 @@
       </c>
       <c r="S178" s="11">
         <f>R178*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B178)</f>
-        <v>800.69545616340542</v>
+        <v>800.69545616337109</v>
       </c>
       <c r="T178" s="11">
         <f t="shared" si="43"/>
-        <v>800.69545616340542</v>
+        <v>800.69545616337109</v>
       </c>
       <c r="U178" s="11">
         <f t="shared" si="44"/>
-        <v>252.2190686914727</v>
+        <v>252.2190686914619</v>
       </c>
       <c r="V178" s="11">
         <f t="shared" si="45"/>
-        <v>1052.9145248548782</v>
+        <v>1052.914524854833</v>
       </c>
       <c r="W178" s="12">
         <f>IF(AND(C178="F",M178&lt;O178,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B178)=1),1,0)</f>
@@ -23812,19 +23812,19 @@
       </c>
       <c r="Z178" s="11">
         <f>Y178*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B178)</f>
-        <v>4141.562799127124</v>
+        <v>4141.5627991270885</v>
       </c>
       <c r="AA178" s="11">
         <f t="shared" si="47"/>
-        <v>4141.562799127124</v>
+        <v>4141.5627991270885</v>
       </c>
       <c r="AB178" s="11">
         <f t="shared" si="48"/>
-        <v>1304.5922817250441</v>
+        <v>1304.592281725033</v>
       </c>
       <c r="AC178" s="11">
         <f t="shared" si="49"/>
-        <v>5446.1550808521679</v>
+        <v>5446.1550808521215</v>
       </c>
       <c r="AD178" s="12">
         <f t="shared" si="50"/>
@@ -23863,7 +23863,7 @@
         <v>1.5</v>
       </c>
       <c r="G179" s="8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H179" s="8">
         <v>1</v>
@@ -23909,19 +23909,19 @@
       </c>
       <c r="S179" s="11">
         <f>R179*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B179)</f>
-        <v>920.42942280932289</v>
+        <v>920.42942280928332</v>
       </c>
       <c r="T179" s="11">
         <f t="shared" si="43"/>
-        <v>920.42942280932289</v>
+        <v>920.42942280928332</v>
       </c>
       <c r="U179" s="11">
         <f t="shared" si="44"/>
-        <v>289.93526818493672</v>
+        <v>289.93526818492427</v>
       </c>
       <c r="V179" s="11">
         <f t="shared" si="45"/>
-        <v>1210.3646909942595</v>
+        <v>1210.3646909942076</v>
       </c>
       <c r="W179" s="12">
         <f>IF(AND(C179="F",M179&lt;O179,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B179)=1),1,0)</f>
@@ -23937,19 +23937,19 @@
       </c>
       <c r="Z179" s="11">
         <f>Y179*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B179)</f>
-        <v>4760.8815903548575</v>
+        <v>4760.8815903548175</v>
       </c>
       <c r="AA179" s="11">
         <f t="shared" si="47"/>
-        <v>4760.8815903548575</v>
+        <v>4760.8815903548175</v>
       </c>
       <c r="AB179" s="11">
         <f t="shared" si="48"/>
-        <v>1499.6777009617801</v>
+        <v>1499.6777009617674</v>
       </c>
       <c r="AC179" s="11">
         <f t="shared" si="49"/>
-        <v>6260.5592913166374</v>
+        <v>6260.5592913165847</v>
       </c>
       <c r="AD179" s="12">
         <f t="shared" si="50"/>
@@ -23988,7 +23988,7 @@
         <v>5.7</v>
       </c>
       <c r="G180" s="8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H180" s="8">
         <v>1</v>
@@ -24034,19 +24034,19 @@
       </c>
       <c r="S180" s="11">
         <f>R180*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B180)</f>
-        <v>568.55282351000733</v>
+        <v>568.55282350998289</v>
       </c>
       <c r="T180" s="11">
         <f t="shared" si="43"/>
-        <v>426.4146176325055</v>
+        <v>426.41461763248719</v>
       </c>
       <c r="U180" s="11">
         <f t="shared" si="44"/>
-        <v>134.32060455423922</v>
+        <v>134.32060455423346</v>
       </c>
       <c r="V180" s="11">
         <f t="shared" si="45"/>
-        <v>560.73522218674475</v>
+        <v>560.73522218672065</v>
       </c>
       <c r="W180" s="12">
         <f>IF(AND(C180="F",M180&lt;O180,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B180)=1),1,0)</f>
@@ -24062,19 +24062,19 @@
       </c>
       <c r="Z180" s="11">
         <f>Y180*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B180)</f>
-        <v>2940.8150190716083</v>
+        <v>2940.8150190715833</v>
       </c>
       <c r="AA180" s="11">
         <f t="shared" si="47"/>
-        <v>2205.6112643037063</v>
+        <v>2205.6112643036877</v>
       </c>
       <c r="AB180" s="11">
         <f t="shared" si="48"/>
-        <v>694.76754825566752</v>
+        <v>694.76754825566161</v>
       </c>
       <c r="AC180" s="11">
         <f t="shared" si="49"/>
-        <v>2900.3788125593737</v>
+        <v>2900.3788125593492</v>
       </c>
       <c r="AD180" s="12">
         <f t="shared" si="50"/>
@@ -24113,7 +24113,7 @@
         <v>9.9</v>
       </c>
       <c r="G181" s="8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H181" s="8">
         <v>1</v>
@@ -24238,7 +24238,7 @@
         <v>5.2</v>
       </c>
       <c r="G182" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H182" s="8">
         <v>1</v>
@@ -24363,7 +24363,7 @@
         <v>9.1999999999999993</v>
       </c>
       <c r="G183" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H183" s="8">
         <v>1</v>
@@ -24488,7 +24488,7 @@
         <v>2.7</v>
       </c>
       <c r="G184" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H184" s="8">
         <v>1</v>
@@ -24613,7 +24613,7 @@
         <v>6.3</v>
       </c>
       <c r="G185" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H185" s="8">
         <v>1</v>
@@ -24738,7 +24738,7 @@
         <v>7.4</v>
       </c>
       <c r="G186" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H186" s="8">
         <v>1</v>
@@ -24863,7 +24863,7 @@
         <v>3.7</v>
       </c>
       <c r="G187" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H187" s="8">
         <v>1</v>
@@ -24988,7 +24988,7 @@
         <v>3.8</v>
       </c>
       <c r="G188" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H188" s="8">
         <v>1</v>
@@ -25113,7 +25113,7 @@
         <v>7.2</v>
       </c>
       <c r="G189" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H189" s="8">
         <v>1</v>
@@ -25238,7 +25238,7 @@
         <v>9.6999999999999993</v>
       </c>
       <c r="G190" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H190" s="8">
         <v>1</v>
@@ -25284,19 +25284,19 @@
       </c>
       <c r="S190" s="11">
         <f>R190*SUMIFS(Categories!$AB$5:$AB$11,Categories!$A$5:$A$11,B190)</f>
-        <v>24.753788103276211</v>
+        <v>24.753788103275149</v>
       </c>
       <c r="T190" s="11">
         <f t="shared" si="43"/>
-        <v>24.753788103276211</v>
+        <v>24.753788103275149</v>
       </c>
       <c r="U190" s="11">
         <f t="shared" si="44"/>
-        <v>7.7974432525320063</v>
+        <v>7.7974432525316715</v>
       </c>
       <c r="V190" s="11">
         <f t="shared" si="45"/>
-        <v>32.55123135580822</v>
+        <v>32.55123135580682</v>
       </c>
       <c r="W190" s="12">
         <f>IF(AND(C190="F",M190&lt;O190,SUMIFS(Categories!$AH$5:$AH$11,Categories!$A$5:$A$11,B190)=1),1,0)</f>
@@ -25312,19 +25312,19 @@
       </c>
       <c r="Z190" s="11">
         <f>Y190*SUMIFS(Categories!$AJ$5:$AJ$11,Categories!$A$5:$A$11,B190)</f>
-        <v>128.03790399565128</v>
+        <v>128.0379039956502</v>
       </c>
       <c r="AA190" s="11">
         <f t="shared" si="47"/>
-        <v>128.03790399565128</v>
+        <v>128.0379039956502</v>
       </c>
       <c r="AB190" s="11">
         <f t="shared" si="48"/>
-        <v>40.331939758630149</v>
+        <v>40.331939758629815</v>
       </c>
       <c r="AC190" s="11">
         <f t="shared" si="49"/>
-        <v>168.36984375428142</v>
+        <v>168.36984375428</v>
       </c>
       <c r="AD190" s="12">
         <f t="shared" si="50"/>
@@ -25363,7 +25363,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="G191" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H191" s="8">
         <v>1</v>
@@ -25488,7 +25488,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="G192" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H192" s="8">
         <v>1</v>
@@ -25613,7 +25613,7 @@
         <v>4</v>
       </c>
       <c r="G193" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H193" s="8">
         <v>1</v>
@@ -25738,7 +25738,7 @@
         <v>4</v>
       </c>
       <c r="G194" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H194" s="8">
         <v>1</v>
@@ -25863,7 +25863,7 @@
         <v>3.2</v>
       </c>
       <c r="G195" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H195" s="8">
         <v>1</v>
@@ -25988,7 +25988,7 @@
         <v>3.2</v>
       </c>
       <c r="G196" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H196" s="8">
         <v>1</v>
@@ -26113,7 +26113,7 @@
         <v>7.1</v>
       </c>
       <c r="G197" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H197" s="8">
         <v>1</v>
@@ -26238,7 +26238,7 @@
         <v>7.1</v>
       </c>
       <c r="G198" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H198" s="8">
         <v>1</v>
@@ -26363,7 +26363,7 @@
         <v>11.9</v>
       </c>
       <c r="G199" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H199" s="8">
         <v>1</v>
@@ -26488,7 +26488,7 @@
         <v>11.9</v>
       </c>
       <c r="G200" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H200" s="8">
         <v>1</v>
@@ -26613,7 +26613,7 @@
         <v>2.4</v>
       </c>
       <c r="G201" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H201" s="8">
         <v>1</v>
@@ -26738,7 +26738,7 @@
         <v>2.4</v>
       </c>
       <c r="G202" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H202" s="8">
         <v>1</v>
@@ -26863,7 +26863,7 @@
         <v>1.7</v>
       </c>
       <c r="G203" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H203" s="8">
         <v>1</v>
@@ -26988,7 +26988,7 @@
         <v>1.7</v>
       </c>
       <c r="G204" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H204" s="8">
         <v>1</v>
@@ -27113,7 +27113,7 @@
         <v>7.3</v>
       </c>
       <c r="G205" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H205" s="8">
         <v>1</v>
@@ -27238,7 +27238,7 @@
         <v>7.3</v>
       </c>
       <c r="G206" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H206" s="8">
         <v>1</v>
@@ -27363,7 +27363,7 @@
         <v>9.6999999999999993</v>
       </c>
       <c r="G207" s="8">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H207" s="8">
         <v>1</v>
@@ -27488,7 +27488,7 @@
         <v>9.6999999999999993</v>
       </c>
       <c r="G208" s="8">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H208" s="8">
         <v>1</v>
@@ -27613,7 +27613,7 @@
         <v>7.8</v>
       </c>
       <c r="G209" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H209" s="8">
         <v>1</v>
@@ -27738,7 +27738,7 @@
         <v>7.8</v>
       </c>
       <c r="G210" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H210" s="8">
         <v>1</v>
@@ -27863,7 +27863,7 @@
         <v>5</v>
       </c>
       <c r="G211" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H211" s="8">
         <v>1</v>
@@ -27988,7 +27988,7 @@
         <v>5</v>
       </c>
       <c r="G212" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H212" s="8">
         <v>1</v>
@@ -28113,7 +28113,7 @@
         <v>11.9</v>
       </c>
       <c r="G213" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H213" s="8">
         <v>1</v>
@@ -28238,7 +28238,7 @@
         <v>11.9</v>
       </c>
       <c r="G214" s="8">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H214" s="8">
         <v>1</v>
@@ -28363,7 +28363,7 @@
         <v>3.7</v>
       </c>
       <c r="G215" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H215" s="8">
         <v>1</v>
@@ -28488,7 +28488,7 @@
         <v>3.7</v>
       </c>
       <c r="G216" s="8">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="H216" s="8">
         <v>1</v>
@@ -28607,7 +28607,8 @@
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="4" width="7" customWidth="1"/>
-    <col min="5" max="63" width="12" customWidth="1"/>
+    <col min="5" max="52" width="12" customWidth="1"/>
+    <col min="53" max="63" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:63" ht="17.399999999999999" x14ac:dyDescent="0.35">
@@ -28863,7 +28864,7 @@
       </c>
       <c r="R5" s="10">
         <f>IF(B5&lt;2,0,SUMPRODUCT((Data!$B$5:$B$216=$A5)*Data!$G$5:$G$216*Data!$G$5:$G$216)/B5-(SUMIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A5)/B5)^2)</f>
-        <v>2.055268595041321</v>
+        <v>2.0552685950413263</v>
       </c>
       <c r="S5" s="10">
         <f>IF(B5&lt;2,0,SUMPRODUCT((Data!$B$5:$B$216=$A5)*Data!$F$5:$F$216*Data!$F$5:$F$216)/B5-(SUMIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A5)/B5)^2)</f>
@@ -28875,23 +28876,23 @@
       </c>
       <c r="U5" s="11">
         <f t="shared" ref="U5:U11" si="5">IF(OR(T5=0,ABS(BK5)&lt;0.000000001),0,((BH5-BB5*BD5/B5)*(BF5-BC5^2/B5)-(BI5-BC5*BD5/B5)*(BG5-BB5*BC5/B5))/BK5)</f>
-        <v>8535.3838587979317</v>
+        <v>8535.3838587976097</v>
       </c>
       <c r="V5" s="11">
         <f t="shared" ref="V5:V11" si="6">IF(OR(T5=0,ABS(BK5)&lt;0.000000001),0,((BI5-BC5*BD5/B5)*(BE5-BB5^2/B5)-(BH5-BB5*BD5/B5)*(BG5-BB5*BC5/B5))/BK5)</f>
-        <v>678.92969527009404</v>
+        <v>678.92969527023718</v>
       </c>
       <c r="W5" s="10">
         <f t="shared" ref="W5:W11" si="7">IF(OR(T5=0,ABS(BK5)&lt;0.000000001,(BJ5-BD5^2/B5)&lt;0.000000001),"",(U5*(BH5-BB5*BD5/B5)+V5*(BI5-BC5*BD5/B5))/(BJ5-BD5^2/B5))</f>
-        <v>0.88827244765407432</v>
+        <v>0.88827244765405566</v>
       </c>
       <c r="X5" s="13">
         <f>IF(H5&gt;=0,MAX(0,MIN(IF(OR(T5=0,E5&lt;=0),0,(U5*(IF(D5=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A5,Data!$C$5:$C$216,"M"))-IF(C5=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A5,Data!$C$5:$C$216,"F")))+V5*(IF(D5=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A5,Data!$C$5:$C$216,"M"))-IF(C5=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A5,Data!$C$5:$C$216,"F"))))/E5*100),H5)),MIN(0,MAX(IF(OR(T5=0,E5&lt;=0),0,(U5*(IF(D5=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A5,Data!$C$5:$C$216,"M"))-IF(C5=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A5,Data!$C$5:$C$216,"F")))+V5*(IF(D5=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A5,Data!$C$5:$C$216,"M"))-IF(C5=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A5,Data!$C$5:$C$216,"F"))))/E5*100),H5)))</f>
-        <v>2.0545467523704719</v>
+        <v>2.0545467523704608</v>
       </c>
       <c r="Y5" s="13">
         <f t="shared" ref="Y5:Y11" si="8">H5-X5</f>
-        <v>9.0800263459079424</v>
+        <v>9.0800263459079531</v>
       </c>
       <c r="Z5" s="12">
         <f t="shared" ref="Z5:Z11" si="9">IF(AND(H5&gt;=0,Y5&gt;threshold_pct),1,0)</f>
@@ -28903,19 +28904,19 @@
       </c>
       <c r="AB5" s="11">
         <f t="shared" ref="AB5:AB11" si="10">IF(Z5=0,0,(Y5-threshold_pct)/100*E5*C5)</f>
-        <v>36567.573492378411</v>
+        <v>36567.573492378506</v>
       </c>
       <c r="AC5" s="11">
         <f>SUMIFS(Data!$T$5:$T$216,Data!$B$5:$B$216,$A5)</f>
-        <v>34928.69603095096</v>
+        <v>34928.696030951061</v>
       </c>
       <c r="AD5" s="11">
         <f>SUMIFS(Data!$U$5:$U$216,Data!$B$5:$B$216,$A5)</f>
-        <v>10874.059110945473</v>
+        <v>10874.059110945502</v>
       </c>
       <c r="AE5" s="11">
         <f t="shared" ref="AE5:AE11" si="11">AC5+AD5</f>
-        <v>45802.755141896429</v>
+        <v>45802.75514189656</v>
       </c>
       <c r="AF5" s="12">
         <f>SUMIFS(Data!$P$5:$P$216,Data!$B$5:$B$216,$A5)</f>
@@ -28923,7 +28924,7 @@
       </c>
       <c r="AG5" s="13">
         <f>IF(E5&lt;=0,0,(E5-(IF(C5=0,0,AVERAGEIFS(Data!$M$5:$M$216,Data!$B$5:$B$216,$A5,Data!$C$5:$C$216,"F"))+IF(C5=0,0,SUMIFS(Data!$S$5:$S$216,Data!$B$5:$B$216,$A5,Data!$C$5:$C$216,"F")/C5)))/E5*100-X5)</f>
-        <v>4.9999999999999929</v>
+        <v>5.0000000000000036</v>
       </c>
       <c r="AH5" s="12">
         <f t="shared" ref="AH5:AH11" si="12">IF(AND(H5&gt;=0,Y5&gt;0),1,0)</f>
@@ -28935,19 +28936,19 @@
       </c>
       <c r="AJ5" s="11">
         <f t="shared" ref="AJ5:AJ11" si="13">IF(AH5=0,0,Y5/100*E5*C5)</f>
-        <v>81380.486929878418</v>
+        <v>81380.48692987852</v>
       </c>
       <c r="AK5" s="11">
         <f>SUMIFS(Data!$AA$5:$AA$216,Data!$B$5:$B$216,$A5)</f>
-        <v>77733.19417589881</v>
+        <v>77733.194175898912</v>
       </c>
       <c r="AL5" s="11">
         <f>SUMIFS(Data!$AB$5:$AB$216,Data!$B$5:$B$216,$A5)</f>
-        <v>20260.687598686683</v>
+        <v>20260.687598686687</v>
       </c>
       <c r="AM5" s="11">
         <f t="shared" ref="AM5:AM11" si="14">AK5+AL5</f>
-        <v>97993.88177458549</v>
+        <v>97993.881774585607</v>
       </c>
       <c r="AN5" s="12">
         <f>SUMIFS(Data!$W$5:$W$216,Data!$B$5:$B$216,$A5)</f>
@@ -28955,7 +28956,7 @@
       </c>
       <c r="AO5" s="13">
         <f>IF(E5&lt;=0,0,(E5-(IF(C5=0,0,AVERAGEIFS(Data!$M$5:$M$216,Data!$B$5:$B$216,$A5,Data!$C$5:$C$216,"F"))+IF(C5=0,0,SUMIFS(Data!$Z$5:$Z$216,Data!$B$5:$B$216,$A5,Data!$C$5:$C$216,"F")/C5)))/E5*100-X5)</f>
-        <v>-7.1054273576010019E-15</v>
+        <v>3.9968028886505635E-15</v>
       </c>
       <c r="AP5" s="12">
         <f t="shared" ref="AP5:AP11" si="15">IF(OR(B5&lt;10,C5&lt;3,D5&lt;3),1,0)</f>
@@ -28971,7 +28972,7 @@
       </c>
       <c r="BB5" s="10">
         <f>SUMIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A5)</f>
-        <v>137</v>
+        <v>401</v>
       </c>
       <c r="BC5" s="10">
         <f>SUMIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A5)</f>
@@ -28983,7 +28984,7 @@
       </c>
       <c r="BE5" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A5)*Data!$G$5:$G$216*Data!$G$5:$G$216)</f>
-        <v>517</v>
+        <v>3745</v>
       </c>
       <c r="BF5" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A5)*Data!$F$5:$F$216*Data!$F$5:$F$216)</f>
@@ -28991,11 +28992,11 @@
       </c>
       <c r="BG5" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A5)*Data!$G$5:$G$216*Data!$F$5:$F$216)</f>
-        <v>1087.1000000000001</v>
+        <v>2917.1</v>
       </c>
       <c r="BH5" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A5)*Data!$G$5:$G$216*Data!$M$5:$M$216)</f>
-        <v>10786741.013333334</v>
+        <v>29905655.733333323</v>
       </c>
       <c r="BI5" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A5)*Data!$F$5:$F$216*Data!$M$5:$M$216)</f>
@@ -29007,7 +29008,7 @@
       </c>
       <c r="BK5" s="10">
         <f t="shared" ref="BK5:BK11" si="18">IF(T5=0,0,((BE5-BB5^2/B5)*(BF5-BC5^2/B5)-(BG5-BB5*BC5/B5)^2))</f>
-        <v>10964.745909090874</v>
+        <v>10964.745909090911</v>
       </c>
     </row>
     <row r="6" spans="1:63" x14ac:dyDescent="0.3">
@@ -29080,7 +29081,7 @@
       </c>
       <c r="R6" s="10">
         <f>IF(B6&lt;2,0,SUMPRODUCT((Data!$B$5:$B$216=$A6)*Data!$G$5:$G$216*Data!$G$5:$G$216)/B6-(SUMIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A6)/B6)^2)</f>
-        <v>2.1724376731301929</v>
+        <v>2.1724376731301902</v>
       </c>
       <c r="S6" s="10">
         <f>IF(B6&lt;2,0,SUMPRODUCT((Data!$B$5:$B$216=$A6)*Data!$F$5:$F$216*Data!$F$5:$F$216)/B6-(SUMIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A6)/B6)^2)</f>
@@ -29092,23 +29093,23 @@
       </c>
       <c r="U6" s="11">
         <f t="shared" si="5"/>
-        <v>7174.9830844705803</v>
+        <v>7174.9830844706439</v>
       </c>
       <c r="V6" s="11">
         <f t="shared" si="6"/>
-        <v>443.77555030723408</v>
+        <v>443.77555030720379</v>
       </c>
       <c r="W6" s="10">
         <f t="shared" si="7"/>
-        <v>0.94277342937722075</v>
+        <v>0.94277342937722619</v>
       </c>
       <c r="X6" s="13">
         <f>IF(H6&gt;=0,MAX(0,MIN(IF(OR(T6=0,E6&lt;=0),0,(U6*(IF(D6=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A6,Data!$C$5:$C$216,"M"))-IF(C6=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A6,Data!$C$5:$C$216,"F")))+V6*(IF(D6=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A6,Data!$C$5:$C$216,"M"))-IF(C6=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A6,Data!$C$5:$C$216,"F"))))/E6*100),H6)),MIN(0,MAX(IF(OR(T6=0,E6&lt;=0),0,(U6*(IF(D6=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A6,Data!$C$5:$C$216,"M"))-IF(C6=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A6,Data!$C$5:$C$216,"F")))+V6*(IF(D6=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A6,Data!$C$5:$C$216,"M"))-IF(C6=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A6,Data!$C$5:$C$216,"F"))))/E6*100),H6)))</f>
-        <v>9.9597136114450837</v>
+        <v>9.9597136114450588</v>
       </c>
       <c r="Y6" s="13">
         <f t="shared" si="8"/>
-        <v>1.4758269694178345</v>
+        <v>1.4758269694178594</v>
       </c>
       <c r="Z6" s="12">
         <f t="shared" si="9"/>
@@ -29140,7 +29141,7 @@
       </c>
       <c r="AG6" s="13">
         <f>IF(E6&lt;=0,0,(E6-(IF(C6=0,0,AVERAGEIFS(Data!$M$5:$M$216,Data!$B$5:$B$216,$A6,Data!$C$5:$C$216,"F"))+IF(C6=0,0,SUMIFS(Data!$S$5:$S$216,Data!$B$5:$B$216,$A6,Data!$C$5:$C$216,"F")/C6)))/E6*100-X6)</f>
-        <v>1.4758269694178345</v>
+        <v>1.4758269694178594</v>
       </c>
       <c r="AH6" s="12">
         <f t="shared" si="12"/>
@@ -29152,19 +29153,19 @@
       </c>
       <c r="AJ6" s="11">
         <f t="shared" si="13"/>
-        <v>16228.186593971279</v>
+        <v>16228.186593971552</v>
       </c>
       <c r="AK6" s="11">
         <f>SUMIFS(Data!$AA$5:$AA$216,Data!$B$5:$B$216,$A6)</f>
-        <v>16228.186593971277</v>
+        <v>16228.18659397155</v>
       </c>
       <c r="AL6" s="11">
         <f>SUMIFS(Data!$AB$5:$AB$216,Data!$B$5:$B$216,$A6)</f>
-        <v>5111.878777100952</v>
+        <v>5111.8787771010384</v>
       </c>
       <c r="AM6" s="11">
         <f t="shared" si="14"/>
-        <v>21340.065371072229</v>
+        <v>21340.065371072589</v>
       </c>
       <c r="AN6" s="12">
         <f>SUMIFS(Data!$W$5:$W$216,Data!$B$5:$B$216,$A6)</f>
@@ -29172,7 +29173,7 @@
       </c>
       <c r="AO6" s="13">
         <f>IF(E6&lt;=0,0,(E6-(IF(C6=0,0,AVERAGEIFS(Data!$M$5:$M$216,Data!$B$5:$B$216,$A6,Data!$C$5:$C$216,"F"))+IF(C6=0,0,SUMIFS(Data!$Z$5:$Z$216,Data!$B$5:$B$216,$A6,Data!$C$5:$C$216,"F")/C6)))/E6*100-X6)</f>
-        <v>5.3290705182007514E-15</v>
+        <v>3.5527136788005009E-15</v>
       </c>
       <c r="AP6" s="12">
         <f t="shared" si="15"/>
@@ -29188,7 +29189,7 @@
       </c>
       <c r="BB6" s="10">
         <f>SUMIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A6)</f>
-        <v>101</v>
+        <v>253</v>
       </c>
       <c r="BC6" s="10">
         <f>SUMIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A6)</f>
@@ -29200,7 +29201,7 @@
       </c>
       <c r="BE6" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A6)*Data!$G$5:$G$216*Data!$G$5:$G$216)</f>
-        <v>351</v>
+        <v>1767</v>
       </c>
       <c r="BF6" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A6)*Data!$F$5:$F$216*Data!$F$5:$F$216)</f>
@@ -29208,11 +29209,11 @@
       </c>
       <c r="BG6" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A6)*Data!$G$5:$G$216*Data!$F$5:$F$216)</f>
-        <v>671.49999999999989</v>
+        <v>1527.5</v>
       </c>
       <c r="BH6" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A6)*Data!$G$5:$G$216*Data!$M$5:$M$216)</f>
-        <v>6148916.4479999999</v>
+        <v>14442732.175333336</v>
       </c>
       <c r="BI6" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A6)*Data!$F$5:$F$216*Data!$M$5:$M$216)</f>
@@ -29224,7 +29225,7 @@
       </c>
       <c r="BK6" s="10">
         <f t="shared" si="18"/>
-        <v>8155.4968421052727</v>
+        <v>8155.4968421052581</v>
       </c>
     </row>
     <row r="7" spans="1:63" x14ac:dyDescent="0.3">
@@ -29309,23 +29310,23 @@
       </c>
       <c r="U7" s="11">
         <f t="shared" si="5"/>
-        <v>12241.047884615467</v>
+        <v>12241.047884615477</v>
       </c>
       <c r="V7" s="11">
         <f t="shared" si="6"/>
-        <v>972.05553580900528</v>
+        <v>972.05553580899607</v>
       </c>
       <c r="W7" s="10">
         <f t="shared" si="7"/>
-        <v>0.90431364612287168</v>
+        <v>0.90431364612287135</v>
       </c>
       <c r="X7" s="13">
         <f>IF(H7&gt;=0,MAX(0,MIN(IF(OR(T7=0,E7&lt;=0),0,(U7*(IF(D7=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A7,Data!$C$5:$C$216,"M"))-IF(C7=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A7,Data!$C$5:$C$216,"F")))+V7*(IF(D7=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A7,Data!$C$5:$C$216,"M"))-IF(C7=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A7,Data!$C$5:$C$216,"F"))))/E7*100),H7)),MIN(0,MAX(IF(OR(T7=0,E7&lt;=0),0,(U7*(IF(D7=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A7,Data!$C$5:$C$216,"M"))-IF(C7=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A7,Data!$C$5:$C$216,"F")))+V7*(IF(D7=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A7,Data!$C$5:$C$216,"M"))-IF(C7=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A7,Data!$C$5:$C$216,"F"))))/E7*100),H7)))</f>
-        <v>8.8851985348742559</v>
+        <v>8.8851985348742772</v>
       </c>
       <c r="Y7" s="13">
         <f t="shared" si="8"/>
-        <v>6.5591192091250754</v>
+        <v>6.5591192091250541</v>
       </c>
       <c r="Z7" s="12">
         <f t="shared" si="9"/>
@@ -29337,19 +29338,19 @@
       </c>
       <c r="AB7" s="11">
         <f t="shared" si="10"/>
-        <v>4346.8960433419461</v>
+        <v>4346.896043341887</v>
       </c>
       <c r="AC7" s="11">
         <f>SUMIFS(Data!$T$5:$T$216,Data!$B$5:$B$216,$A7)</f>
-        <v>4346.8960433419461</v>
+        <v>4346.896043341887</v>
       </c>
       <c r="AD7" s="11">
         <f>SUMIFS(Data!$U$5:$U$216,Data!$B$5:$B$216,$A7)</f>
-        <v>41.730202016082671</v>
+        <v>41.73020201608211</v>
       </c>
       <c r="AE7" s="11">
         <f t="shared" si="11"/>
-        <v>4388.6262453580284</v>
+        <v>4388.6262453579693</v>
       </c>
       <c r="AF7" s="12">
         <f>SUMIFS(Data!$P$5:$P$216,Data!$B$5:$B$216,$A7)</f>
@@ -29357,7 +29358,7 @@
       </c>
       <c r="AG7" s="13">
         <f>IF(E7&lt;=0,0,(E7-(IF(C7=0,0,AVERAGEIFS(Data!$M$5:$M$216,Data!$B$5:$B$216,$A7,Data!$C$5:$C$216,"F"))+IF(C7=0,0,SUMIFS(Data!$S$5:$S$216,Data!$B$5:$B$216,$A7,Data!$C$5:$C$216,"F")/C7)))/E7*100-X7)</f>
-        <v>5.0000000000000071</v>
+        <v>5</v>
       </c>
       <c r="AH7" s="12">
         <f t="shared" si="12"/>
@@ -29369,19 +29370,19 @@
       </c>
       <c r="AJ7" s="11">
         <f t="shared" si="13"/>
-        <v>18287.125943341947</v>
+        <v>18287.125943341889</v>
       </c>
       <c r="AK7" s="11">
         <f>SUMIFS(Data!$AA$5:$AA$216,Data!$B$5:$B$216,$A7)</f>
-        <v>18287.125943341947</v>
+        <v>18287.125943341889</v>
       </c>
       <c r="AL7" s="11">
         <f>SUMIFS(Data!$AB$5:$AB$216,Data!$B$5:$B$216,$A7)</f>
-        <v>175.55640905608271</v>
+        <v>175.55640905608212</v>
       </c>
       <c r="AM7" s="11">
         <f t="shared" si="14"/>
-        <v>18462.682352398031</v>
+        <v>18462.682352397973</v>
       </c>
       <c r="AN7" s="12">
         <f>SUMIFS(Data!$W$5:$W$216,Data!$B$5:$B$216,$A7)</f>
@@ -29389,7 +29390,7 @@
       </c>
       <c r="AO7" s="13">
         <f>IF(E7&lt;=0,0,(E7-(IF(C7=0,0,AVERAGEIFS(Data!$M$5:$M$216,Data!$B$5:$B$216,$A7,Data!$C$5:$C$216,"F"))+IF(C7=0,0,SUMIFS(Data!$Z$5:$Z$216,Data!$B$5:$B$216,$A7,Data!$C$5:$C$216,"F")/C7)))/E7*100-X7)</f>
-        <v>5.3290705182007514E-15</v>
+        <v>0</v>
       </c>
       <c r="AP7" s="12">
         <f t="shared" si="15"/>
@@ -29405,7 +29406,7 @@
       </c>
       <c r="BB7" s="10">
         <f>SUMIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A7)</f>
-        <v>33</v>
+        <v>81</v>
       </c>
       <c r="BC7" s="10">
         <f>SUMIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A7)</f>
@@ -29417,7 +29418,7 @@
       </c>
       <c r="BE7" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A7)*Data!$G$5:$G$216*Data!$G$5:$G$216)</f>
-        <v>143</v>
+        <v>827</v>
       </c>
       <c r="BF7" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A7)*Data!$F$5:$F$216*Data!$F$5:$F$216)</f>
@@ -29425,11 +29426,11 @@
       </c>
       <c r="BG7" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A7)*Data!$G$5:$G$216*Data!$F$5:$F$216)</f>
-        <v>195.1</v>
+        <v>465.7</v>
       </c>
       <c r="BH7" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A7)*Data!$G$5:$G$216*Data!$M$5:$M$216)</f>
-        <v>2982196.7300000004</v>
+        <v>7184713.4900000002</v>
       </c>
       <c r="BI7" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A7)*Data!$F$5:$F$216*Data!$M$5:$M$216)</f>
@@ -29441,7 +29442,7 @@
       </c>
       <c r="BK7" s="10">
         <f t="shared" si="18"/>
-        <v>235.62500000000006</v>
+        <v>235.62499999999955</v>
       </c>
     </row>
     <row r="8" spans="1:63" x14ac:dyDescent="0.3">
@@ -29514,7 +29515,7 @@
       </c>
       <c r="R8" s="10">
         <f>IF(B8&lt;2,0,SUMPRODUCT((Data!$B$5:$B$216=$A8)*Data!$G$5:$G$216*Data!$G$5:$G$216)/B8-(SUMIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A8)/B8)^2)</f>
-        <v>1.705621301775146</v>
+        <v>1.7056213017751531</v>
       </c>
       <c r="S8" s="10">
         <f>IF(B8&lt;2,0,SUMPRODUCT((Data!$B$5:$B$216=$A8)*Data!$F$5:$F$216*Data!$F$5:$F$216)/B8-(SUMIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A8)/B8)^2)</f>
@@ -29526,7 +29527,7 @@
       </c>
       <c r="U8" s="11">
         <f t="shared" si="5"/>
-        <v>6673.9272922689588</v>
+        <v>6673.9272922689715</v>
       </c>
       <c r="V8" s="11">
         <f t="shared" si="6"/>
@@ -29534,15 +29535,15 @@
       </c>
       <c r="W8" s="10">
         <f t="shared" si="7"/>
-        <v>0.8747952313048909</v>
+        <v>0.87479523130489234</v>
       </c>
       <c r="X8" s="13">
         <f>IF(H8&gt;=0,MAX(0,MIN(IF(OR(T8=0,E8&lt;=0),0,(U8*(IF(D8=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A8,Data!$C$5:$C$216,"M"))-IF(C8=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A8,Data!$C$5:$C$216,"F")))+V8*(IF(D8=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A8,Data!$C$5:$C$216,"M"))-IF(C8=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A8,Data!$C$5:$C$216,"F"))))/E8*100),H8)),MIN(0,MAX(IF(OR(T8=0,E8&lt;=0),0,(U8*(IF(D8=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A8,Data!$C$5:$C$216,"M"))-IF(C8=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A8,Data!$C$5:$C$216,"F")))+V8*(IF(D8=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A8,Data!$C$5:$C$216,"M"))-IF(C8=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A8,Data!$C$5:$C$216,"F"))))/E8*100),H8)))</f>
-        <v>-6.3388453946482866</v>
+        <v>-6.3388453946482946</v>
       </c>
       <c r="Y8" s="13">
         <f t="shared" si="8"/>
-        <v>-7.299683194235369</v>
+        <v>-7.2996831942353611</v>
       </c>
       <c r="Z8" s="12">
         <f t="shared" si="9"/>
@@ -29574,7 +29575,7 @@
       </c>
       <c r="AG8" s="13">
         <f>IF(E8&lt;=0,0,(E8-(IF(C8=0,0,AVERAGEIFS(Data!$M$5:$M$216,Data!$B$5:$B$216,$A8,Data!$C$5:$C$216,"F"))+IF(C8=0,0,SUMIFS(Data!$S$5:$S$216,Data!$B$5:$B$216,$A8,Data!$C$5:$C$216,"F")/C8)))/E8*100-X8)</f>
-        <v>-7.299683194235369</v>
+        <v>-7.2996831942353611</v>
       </c>
       <c r="AH8" s="12">
         <f t="shared" si="12"/>
@@ -29606,7 +29607,7 @@
       </c>
       <c r="AO8" s="13">
         <f>IF(E8&lt;=0,0,(E8-(IF(C8=0,0,AVERAGEIFS(Data!$M$5:$M$216,Data!$B$5:$B$216,$A8,Data!$C$5:$C$216,"F"))+IF(C8=0,0,SUMIFS(Data!$Z$5:$Z$216,Data!$B$5:$B$216,$A8,Data!$C$5:$C$216,"F")/C8)))/E8*100-X8)</f>
-        <v>-7.299683194235369</v>
+        <v>-7.2996831942353611</v>
       </c>
       <c r="AP8" s="12">
         <f t="shared" si="15"/>
@@ -29622,7 +29623,7 @@
       </c>
       <c r="BB8" s="10">
         <f>SUMIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A8)</f>
-        <v>93</v>
+        <v>223</v>
       </c>
       <c r="BC8" s="10">
         <f>SUMIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A8)</f>
@@ -29634,7 +29635,7 @@
       </c>
       <c r="BE8" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A8)*Data!$G$5:$G$216*Data!$G$5:$G$216)</f>
-        <v>377</v>
+        <v>1957</v>
       </c>
       <c r="BF8" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A8)*Data!$F$5:$F$216*Data!$F$5:$F$216)</f>
@@ -29642,11 +29643,11 @@
       </c>
       <c r="BG8" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A8)*Data!$G$5:$G$216*Data!$F$5:$F$216)</f>
-        <v>800.19999999999993</v>
+        <v>1821.6999999999998</v>
       </c>
       <c r="BH8" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A8)*Data!$G$5:$G$216*Data!$M$5:$M$216)</f>
-        <v>7116799.5100000007</v>
+        <v>16567940.109999999</v>
       </c>
       <c r="BI8" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A8)*Data!$F$5:$F$216*Data!$M$5:$M$216)</f>
@@ -29658,7 +29659,7 @@
       </c>
       <c r="BK8" s="10">
         <f t="shared" si="18"/>
-        <v>3597.6615384615507</v>
+        <v>3597.6615384615552</v>
       </c>
     </row>
     <row r="9" spans="1:63" x14ac:dyDescent="0.3">
@@ -29731,7 +29732,7 @@
       </c>
       <c r="R9" s="10">
         <f>IF(B9&lt;2,0,SUMPRODUCT((Data!$B$5:$B$216=$A9)*Data!$G$5:$G$216*Data!$G$5:$G$216)/B9-(SUMIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A9)/B9)^2)</f>
-        <v>1.5875000000000004</v>
+        <v>1.5874999999999986</v>
       </c>
       <c r="S9" s="10">
         <f>IF(B9&lt;2,0,SUMPRODUCT((Data!$B$5:$B$216=$A9)*Data!$F$5:$F$216*Data!$F$5:$F$216)/B9-(SUMIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A9)/B9)^2)</f>
@@ -29743,23 +29744,23 @@
       </c>
       <c r="U9" s="11">
         <f t="shared" si="5"/>
-        <v>5756.2949399498621</v>
+        <v>5756.2949399499039</v>
       </c>
       <c r="V9" s="11">
         <f t="shared" si="6"/>
-        <v>727.89015666116052</v>
+        <v>727.89015666114597</v>
       </c>
       <c r="W9" s="10">
         <f t="shared" si="7"/>
-        <v>0.91301296861931103</v>
+        <v>0.91301296861931192</v>
       </c>
       <c r="X9" s="13">
         <f>IF(H9&gt;=0,MAX(0,MIN(IF(OR(T9=0,E9&lt;=0),0,(U9*(IF(D9=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A9,Data!$C$5:$C$216,"M"))-IF(C9=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A9,Data!$C$5:$C$216,"F")))+V9*(IF(D9=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A9,Data!$C$5:$C$216,"M"))-IF(C9=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A9,Data!$C$5:$C$216,"F"))))/E9*100),H9)),MIN(0,MAX(IF(OR(T9=0,E9&lt;=0),0,(U9*(IF(D9=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A9,Data!$C$5:$C$216,"M"))-IF(C9=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A9,Data!$C$5:$C$216,"F")))+V9*(IF(D9=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A9,Data!$C$5:$C$216,"M"))-IF(C9=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A9,Data!$C$5:$C$216,"F"))))/E9*100),H9)))</f>
-        <v>8.9498183217178582</v>
+        <v>8.9498183217178298</v>
       </c>
       <c r="Y9" s="13">
         <f t="shared" si="8"/>
-        <v>6.6592510343695288</v>
+        <v>6.6592510343695572</v>
       </c>
       <c r="Z9" s="12">
         <f t="shared" si="9"/>
@@ -29771,19 +29772,19 @@
       </c>
       <c r="AB9" s="11">
         <f t="shared" si="10"/>
-        <v>17116.569999764306</v>
+        <v>17116.569999764601</v>
       </c>
       <c r="AC9" s="11">
         <f>SUMIFS(Data!$T$5:$T$216,Data!$B$5:$B$216,$A9)</f>
-        <v>16438.891717589966</v>
+        <v>16438.891717590253</v>
       </c>
       <c r="AD9" s="11">
         <f>SUMIFS(Data!$U$5:$U$216,Data!$B$5:$B$216,$A9)</f>
-        <v>5178.2508910408396</v>
+        <v>5178.2508910409288</v>
       </c>
       <c r="AE9" s="11">
         <f t="shared" si="11"/>
-        <v>21617.142608630806</v>
+        <v>21617.142608631184</v>
       </c>
       <c r="AF9" s="12">
         <f>SUMIFS(Data!$P$5:$P$216,Data!$B$5:$B$216,$A9)</f>
@@ -29791,7 +29792,7 @@
       </c>
       <c r="AG9" s="13">
         <f>IF(E9&lt;=0,0,(E9-(IF(C9=0,0,AVERAGEIFS(Data!$M$5:$M$216,Data!$B$5:$B$216,$A9,Data!$C$5:$C$216,"F"))+IF(C9=0,0,SUMIFS(Data!$S$5:$S$216,Data!$B$5:$B$216,$A9,Data!$C$5:$C$216,"F")/C9)))/E9*100-X9)</f>
-        <v>5</v>
+        <v>5.0000000000000036</v>
       </c>
       <c r="AH9" s="12">
         <f t="shared" si="12"/>
@@ -29803,19 +29804,19 @@
       </c>
       <c r="AJ9" s="11">
         <f t="shared" si="13"/>
-        <v>68695.775452145259</v>
+        <v>68695.77545214555</v>
       </c>
       <c r="AK9" s="11">
         <f>SUMIFS(Data!$AA$5:$AA$216,Data!$B$5:$B$216,$A9)</f>
-        <v>65975.976152303949</v>
+        <v>65975.976152304211</v>
       </c>
       <c r="AL9" s="11">
         <f>SUMIFS(Data!$AB$5:$AB$216,Data!$B$5:$B$216,$A9)</f>
-        <v>20782.432487975744</v>
+        <v>20782.432487975828</v>
       </c>
       <c r="AM9" s="11">
         <f t="shared" si="14"/>
-        <v>86758.408640279697</v>
+        <v>86758.408640280046</v>
       </c>
       <c r="AN9" s="12">
         <f>SUMIFS(Data!$W$5:$W$216,Data!$B$5:$B$216,$A9)</f>
@@ -29823,7 +29824,7 @@
       </c>
       <c r="AO9" s="13">
         <f>IF(E9&lt;=0,0,(E9-(IF(C9=0,0,AVERAGEIFS(Data!$M$5:$M$216,Data!$B$5:$B$216,$A9,Data!$C$5:$C$216,"F"))+IF(C9=0,0,SUMIFS(Data!$Z$5:$Z$216,Data!$B$5:$B$216,$A9,Data!$C$5:$C$216,"F")/C9)))/E9*100-X9)</f>
-        <v>0</v>
+        <v>3.5527136788005009E-15</v>
       </c>
       <c r="AP9" s="12">
         <f t="shared" si="15"/>
@@ -29839,7 +29840,7 @@
       </c>
       <c r="BB9" s="10">
         <f>SUMIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A9)</f>
-        <v>110</v>
+        <v>230</v>
       </c>
       <c r="BC9" s="10">
         <f>SUMIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A9)</f>
@@ -29851,7 +29852,7 @@
       </c>
       <c r="BE9" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A9)*Data!$G$5:$G$216*Data!$G$5:$G$216)</f>
-        <v>366</v>
+        <v>1386</v>
       </c>
       <c r="BF9" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A9)*Data!$F$5:$F$216*Data!$F$5:$F$216)</f>
@@ -29859,11 +29860,11 @@
       </c>
       <c r="BG9" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A9)*Data!$G$5:$G$216*Data!$F$5:$F$216)</f>
-        <v>1293.6999999999998</v>
+        <v>2527.0000000000005</v>
       </c>
       <c r="BH9" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A9)*Data!$G$5:$G$216*Data!$M$5:$M$216)</f>
-        <v>6013820.3900000006</v>
+        <v>12046026.410000002</v>
       </c>
       <c r="BI9" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A9)*Data!$F$5:$F$216*Data!$M$5:$M$216)</f>
@@ -29875,7 +29876,7 @@
       </c>
       <c r="BK9" s="10">
         <f t="shared" si="18"/>
-        <v>22741.978500000117</v>
+        <v>22741.978499999896</v>
       </c>
     </row>
     <row r="10" spans="1:63" x14ac:dyDescent="0.3">
@@ -29960,23 +29961,23 @@
       </c>
       <c r="U10" s="11">
         <f t="shared" si="5"/>
-        <v>4902.1583171688662</v>
+        <v>4902.1583171689235</v>
       </c>
       <c r="V10" s="11">
         <f t="shared" si="6"/>
-        <v>472.83278671394805</v>
+        <v>472.83278671392975</v>
       </c>
       <c r="W10" s="10">
         <f t="shared" si="7"/>
-        <v>0.89580044604282516</v>
+        <v>0.89580044604282905</v>
       </c>
       <c r="X10" s="13">
         <f>IF(H10&gt;=0,MAX(0,MIN(IF(OR(T10=0,E10&lt;=0),0,(U10*(IF(D10=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A10,Data!$C$5:$C$216,"M"))-IF(C10=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A10,Data!$C$5:$C$216,"F")))+V10*(IF(D10=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A10,Data!$C$5:$C$216,"M"))-IF(C10=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A10,Data!$C$5:$C$216,"F"))))/E10*100),H10)),MIN(0,MAX(IF(OR(T10=0,E10&lt;=0),0,(U10*(IF(D10=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A10,Data!$C$5:$C$216,"M"))-IF(C10=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A10,Data!$C$5:$C$216,"F")))+V10*(IF(D10=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A10,Data!$C$5:$C$216,"M"))-IF(C10=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A10,Data!$C$5:$C$216,"F"))))/E10*100),H10)))</f>
-        <v>10.837511742810863</v>
+        <v>10.837511742810914</v>
       </c>
       <c r="Y10" s="13">
         <f t="shared" si="8"/>
-        <v>6.1983347046834556</v>
+        <v>6.1983347046834041</v>
       </c>
       <c r="Z10" s="12">
         <f t="shared" si="9"/>
@@ -29988,19 +29989,19 @@
       </c>
       <c r="AB10" s="11">
         <f t="shared" si="10"/>
-        <v>6631.7908758775702</v>
+        <v>6631.7908758772855</v>
       </c>
       <c r="AC10" s="11">
         <f>SUMIFS(Data!$T$5:$T$216,Data!$B$5:$B$216,$A10)</f>
-        <v>6181.8028679851186</v>
+        <v>6181.8028679848521</v>
       </c>
       <c r="AD10" s="11">
         <f>SUMIFS(Data!$U$5:$U$216,Data!$B$5:$B$216,$A10)</f>
-        <v>1947.267903415312</v>
+        <v>1947.2679034152284</v>
       </c>
       <c r="AE10" s="11">
         <f t="shared" si="11"/>
-        <v>8129.0707714004311</v>
+        <v>8129.07077140008</v>
       </c>
       <c r="AF10" s="12">
         <f>SUMIFS(Data!$P$5:$P$216,Data!$B$5:$B$216,$A10)</f>
@@ -30008,7 +30009,7 @@
       </c>
       <c r="AG10" s="13">
         <f>IF(E10&lt;=0,0,(E10-(IF(C10=0,0,AVERAGEIFS(Data!$M$5:$M$216,Data!$B$5:$B$216,$A10,Data!$C$5:$C$216,"F"))+IF(C10=0,0,SUMIFS(Data!$S$5:$S$216,Data!$B$5:$B$216,$A10,Data!$C$5:$C$216,"F")/C10)))/E10*100-X10)</f>
-        <v>5.0000000000000018</v>
+        <v>5</v>
       </c>
       <c r="AH10" s="12">
         <f t="shared" si="12"/>
@@ -30020,19 +30021,19 @@
       </c>
       <c r="AJ10" s="11">
         <f t="shared" si="13"/>
-        <v>34302.652989603062</v>
+        <v>34302.652989602771</v>
       </c>
       <c r="AK10" s="11">
         <f>SUMIFS(Data!$AA$5:$AA$216,Data!$B$5:$B$216,$A10)</f>
-        <v>31975.109378364716</v>
+        <v>31975.109378364446</v>
       </c>
       <c r="AL10" s="11">
         <f>SUMIFS(Data!$AB$5:$AB$216,Data!$B$5:$B$216,$A10)</f>
-        <v>10072.159454184888</v>
+        <v>10072.159454184803</v>
       </c>
       <c r="AM10" s="11">
         <f t="shared" si="14"/>
-        <v>42047.268832549606</v>
+        <v>42047.268832549249</v>
       </c>
       <c r="AN10" s="12">
         <f>SUMIFS(Data!$W$5:$W$216,Data!$B$5:$B$216,$A10)</f>
@@ -30056,7 +30057,7 @@
       </c>
       <c r="BB10" s="10">
         <f>SUMIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A10)</f>
-        <v>69</v>
+        <v>129</v>
       </c>
       <c r="BC10" s="10">
         <f>SUMIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A10)</f>
@@ -30068,7 +30069,7 @@
       </c>
       <c r="BE10" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A10)*Data!$G$5:$G$216*Data!$G$5:$G$216)</f>
-        <v>193</v>
+        <v>589</v>
       </c>
       <c r="BF10" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A10)*Data!$F$5:$F$216*Data!$F$5:$F$216)</f>
@@ -30076,11 +30077,11 @@
       </c>
       <c r="BG10" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A10)*Data!$G$5:$G$216*Data!$F$5:$F$216)</f>
-        <v>510.89999999999992</v>
+        <v>893.09999999999991</v>
       </c>
       <c r="BH10" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A10)*Data!$G$5:$G$216*Data!$M$5:$M$216)</f>
-        <v>2922416.1293333336</v>
+        <v>5288090.932000001</v>
       </c>
       <c r="BI10" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A10)*Data!$F$5:$F$216*Data!$M$5:$M$216)</f>
@@ -30092,7 +30093,7 @@
       </c>
       <c r="BK10" s="10">
         <f t="shared" si="18"/>
-        <v>3780.5220000000172</v>
+        <v>3780.5219999999863</v>
       </c>
     </row>
     <row r="11" spans="1:63" x14ac:dyDescent="0.3">
@@ -30165,7 +30166,7 @@
       </c>
       <c r="R11" s="10">
         <f>IF(B11&lt;2,0,SUMPRODUCT((Data!$B$5:$B$216=$A11)*Data!$G$5:$G$216*Data!$G$5:$G$216)/B11-(SUMIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A11)/B11)^2)</f>
-        <v>1.5976331360946716</v>
+        <v>1.5976331360946858</v>
       </c>
       <c r="S11" s="10">
         <f>IF(B11&lt;2,0,SUMPRODUCT((Data!$B$5:$B$216=$A11)*Data!$F$5:$F$216*Data!$F$5:$F$216)/B11-(SUMIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A11)/B11)^2)</f>
@@ -30177,15 +30178,15 @@
       </c>
       <c r="U11" s="11">
         <f t="shared" si="5"/>
-        <v>9853.8891175893277</v>
+        <v>9853.8891175898862</v>
       </c>
       <c r="V11" s="11">
         <f t="shared" si="6"/>
-        <v>1314.982287978715</v>
+        <v>1314.9822879785131</v>
       </c>
       <c r="W11" s="10">
         <f t="shared" si="7"/>
-        <v>0.91376832136089492</v>
+        <v>0.91376832136090436</v>
       </c>
       <c r="X11" s="13">
         <f>IF(H11&gt;=0,MAX(0,MIN(IF(OR(T11=0,E11&lt;=0),0,(U11*(IF(D11=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A11,Data!$C$5:$C$216,"M"))-IF(C11=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A11,Data!$C$5:$C$216,"F")))+V11*(IF(D11=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A11,Data!$C$5:$C$216,"M"))-IF(C11=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A11,Data!$C$5:$C$216,"F"))))/E11*100),H11)),MIN(0,MAX(IF(OR(T11=0,E11&lt;=0),0,(U11*(IF(D11=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A11,Data!$C$5:$C$216,"M"))-IF(C11=0,0,AVERAGEIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A11,Data!$C$5:$C$216,"F")))+V11*(IF(D11=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A11,Data!$C$5:$C$216,"M"))-IF(C11=0,0,AVERAGEIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A11,Data!$C$5:$C$216,"F"))))/E11*100),H11)))</f>
@@ -30273,7 +30274,7 @@
       </c>
       <c r="BB11" s="10">
         <f>SUMIFS(Data!$G$5:$G$216,Data!$B$5:$B$216,$A11)</f>
-        <v>96</v>
+        <v>252</v>
       </c>
       <c r="BC11" s="10">
         <f>SUMIFS(Data!$F$5:$F$216,Data!$B$5:$B$216,$A11)</f>
@@ -30285,7 +30286,7 @@
       </c>
       <c r="BE11" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A11)*Data!$G$5:$G$216*Data!$G$5:$G$216)</f>
-        <v>396</v>
+        <v>2484</v>
       </c>
       <c r="BF11" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A11)*Data!$F$5:$F$216*Data!$F$5:$F$216)</f>
@@ -30293,11 +30294,11 @@
       </c>
       <c r="BG11" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A11)*Data!$G$5:$G$216*Data!$F$5:$F$216)</f>
-        <v>686.2</v>
+        <v>1647.4</v>
       </c>
       <c r="BH11" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A11)*Data!$G$5:$G$216*Data!$M$5:$M$216)</f>
-        <v>9018458.3600000013</v>
+        <v>22805972.780000005</v>
       </c>
       <c r="BI11" s="10">
         <f>SUMPRODUCT((Data!$B$5:$B$216=$A11)*Data!$F$5:$F$216*Data!$M$5:$M$216)</f>
@@ -30309,7 +30310,7 @@
       </c>
       <c r="BK11" s="10">
         <f t="shared" si="18"/>
-        <v>2768.0461538461695</v>
+        <v>2768.0461538460731</v>
       </c>
     </row>
   </sheetData>
@@ -30374,15 +30375,15 @@
       </c>
       <c r="B8" s="11">
         <f>SUM(Categories!$AC$5:$AC$11)</f>
-        <v>126314.95415986807</v>
+        <v>126314.95415986812</v>
       </c>
       <c r="C8" s="11">
         <f>SUM(Categories!$AK$5:$AK$11)</f>
-        <v>335191.02224388078</v>
+        <v>335191.02224388107</v>
       </c>
       <c r="D8" s="11">
         <f t="shared" ref="D8:D14" si="0">C8-B8</f>
-        <v>208876.06808401272</v>
+        <v>208876.06808401295</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -30391,15 +30392,15 @@
       </c>
       <c r="B9" s="11">
         <f>SUM(Categories!$AD$5:$AD$11)</f>
-        <v>22110.594615417707</v>
+        <v>22110.594615417744</v>
       </c>
       <c r="C9" s="11">
         <f>SUM(Categories!$AL$5:$AL$11)</f>
-        <v>61053.499755004348</v>
+        <v>61053.499755004435</v>
       </c>
       <c r="D9" s="11">
         <f t="shared" si="0"/>
-        <v>38942.905139586641</v>
+        <v>38942.905139586692</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -30408,15 +30409,15 @@
       </c>
       <c r="B10" s="17">
         <f>B8+B9</f>
-        <v>148425.54877528577</v>
+        <v>148425.54877528586</v>
       </c>
       <c r="C10" s="17">
         <f>C8+C9</f>
-        <v>396244.52199888515</v>
+        <v>396244.5219988855</v>
       </c>
       <c r="D10" s="17">
         <f t="shared" si="0"/>
-        <v>247818.97322359937</v>
+        <v>247818.97322359963</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -30425,15 +30426,15 @@
       </c>
       <c r="B11" s="13">
         <f>IF($B$4=0,0,B10/$B$4*100)</f>
-        <v>1.1392167947939389</v>
+        <v>1.1392167947939396</v>
       </c>
       <c r="C11" s="13">
         <f>IF($B$4=0,0,C10/$B$4*100)</f>
-        <v>3.041312078890491</v>
+        <v>3.0413120788904937</v>
       </c>
       <c r="D11" s="13">
         <f t="shared" si="0"/>
-        <v>1.9020952840965522</v>
+        <v>1.9020952840965542</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -30459,15 +30460,15 @@
       </c>
       <c r="B13" s="11">
         <f>B10*(13-implementation_month)/12</f>
-        <v>74212.774387642887</v>
+        <v>74212.77438764293</v>
       </c>
       <c r="C13" s="11">
         <f>C10*(13-implementation_month)/12</f>
-        <v>198122.26099944257</v>
+        <v>198122.26099944275</v>
       </c>
       <c r="D13" s="11">
         <f t="shared" si="0"/>
-        <v>123909.48661179969</v>
+        <v>123909.48661179982</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -30476,15 +30477,15 @@
       </c>
       <c r="B14" s="11">
         <f>B10</f>
-        <v>148425.54877528577</v>
+        <v>148425.54877528586</v>
       </c>
       <c r="C14" s="11">
         <f>C10</f>
-        <v>396244.52199888515</v>
+        <v>396244.5219988855</v>
       </c>
       <c r="D14" s="11">
         <f t="shared" si="0"/>
-        <v>247818.97322359937</v>
+        <v>247818.97322359963</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>